<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 11/08/2026 06:50:38
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1974</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1974</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1003,12 +1003,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1974</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1089,22 +1089,22 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1195,12 +1195,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -1217,22 +1217,22 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1974</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1803,12 +1803,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1995,12 +1995,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2187,12 +2187,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2379,12 +2379,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2507,12 +2507,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>210726125342825</t>
+          <t>210726125342857</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>210726125342857</t>
+          <t>210726125342810</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>210726125342810</t>
+          <t>210726125342779</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>210726125342779</t>
+          <t>210726125342888</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>210726125342888</t>
+          <t>210726125342872</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>210726125342872</t>
+          <t>210726125342716</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>24</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2955,12 +2955,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>210726125342716</t>
+          <t>210726125342763</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>210726125342763</t>
+          <t>210726125342825</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3499,12 +3499,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CAL-027-001-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -3521,27 +3521,27 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132439966</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3563,12 +3563,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-001-002</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -3585,27 +3585,27 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439966</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3627,12 +3627,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132440497</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3691,12 +3691,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132440497</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -5377,22 +5377,22 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5505,22 +5505,22 @@
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -6145,12 +6145,12 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6209,12 +6209,12 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7499,12 +7499,12 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7553,12 +7553,12 @@
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7627,12 +7627,12 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7681,12 +7681,12 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7809,12 +7809,12 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7873,12 +7873,12 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7915,12 +7915,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C118" t="inlineStr"/>
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8043,12 +8043,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8171,12 +8171,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8235,12 +8235,12 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C123" t="inlineStr"/>
@@ -8272,7 +8272,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8331,12 +8331,12 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -8395,12 +8395,12 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8491,12 +8491,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8833,22 +8833,22 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9003,12 +9003,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9131,12 +9131,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9473,22 +9473,22 @@
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -10123,12 +10123,12 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -10251,12 +10251,12 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -10320,7 +10320,7 @@
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10768,7 +10768,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>200226062756258</t>
+          <t>200226070819709</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>200226070819709</t>
+          <t>200226062756258</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>050826061104264</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -11009,12 +11009,12 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050526131349498</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>050526131349498</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>050826061104264</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11531,12 +11531,12 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11777,12 +11777,12 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11792,7 +11792,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11851,12 +11851,12 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -11920,7 +11920,7 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>200226062905996</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11984,7 +11984,7 @@
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226062905996</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -12016,7 +12016,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C182" t="inlineStr"/>
@@ -12033,22 +12033,22 @@
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
@@ -12097,22 +12097,22 @@
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12299,12 +12299,12 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12336,7 +12336,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
@@ -12353,22 +12353,22 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12400,7 +12400,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12555,12 +12555,12 @@
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12619,12 +12619,12 @@
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12673,22 +12673,22 @@
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -12737,22 +12737,22 @@
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12929,22 +12929,22 @@
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1958</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -12959,7 +12959,7 @@
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N196" t="inlineStr">
@@ -12993,22 +12993,22 @@
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1958</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13023,7 +13023,7 @@
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N197" t="inlineStr">
@@ -13067,12 +13067,12 @@
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -13087,7 +13087,7 @@
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N198" t="inlineStr">
@@ -13131,12 +13131,12 @@
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>44</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13151,7 +13151,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>44</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>300726064012575</t>
+          <t>300726064012668</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>300726064011997</t>
+          <t>300726064012684</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>300726064013043</t>
+          <t>300726064012637</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>300726064012668</t>
+          <t>300726064012512</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>300726064012684</t>
+          <t>300726064011997</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>300726064012637</t>
+          <t>300726064013043</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>300726064012512</t>
+          <t>300726064011965</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>300726064011903</t>
+          <t>300726064012575</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>300726064011887</t>
+          <t>300726064011903</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>300726064012809</t>
+          <t>300726064011981</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>300726064011965</t>
+          <t>300726064011887</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14064,7 +14064,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C214" t="inlineStr"/>
@@ -14081,12 +14081,12 @@
       <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>1988</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>300726064012028</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>300726064012543</t>
+          <t>300726064012028</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>300726064011981</t>
+          <t>300726064012981</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>300726064012653</t>
+          <t>300726064012543</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>300726064012497</t>
+          <t>300726064012793</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -14416,7 +14416,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>300726064012793</t>
+          <t>300726064011918</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>300726064011918</t>
+          <t>300726064012012</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14512,7 +14512,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C221" t="inlineStr"/>
@@ -14529,12 +14529,12 @@
       <c r="F221" t="inlineStr"/>
       <c r="G221" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1988</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>300726064012809</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -14576,7 +14576,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C222" t="inlineStr"/>
@@ -14593,22 +14593,22 @@
       <c r="F222" t="inlineStr"/>
       <c r="G222" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>1988</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>300726064012887</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -14623,7 +14623,7 @@
       </c>
       <c r="M222" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N222" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>300726064012981</t>
+          <t>300726064012731</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>300726064012528</t>
+          <t>300726064012590</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>300726064013028</t>
+          <t>300726064012700</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>300726064012965</t>
+          <t>300726064012653</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14928,7 +14928,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>300726064011934</t>
+          <t>300726064011950</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -14992,7 +14992,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>300726064012012</t>
+          <t>300726064012497</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -15024,7 +15024,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C229" t="inlineStr"/>
@@ -15041,22 +15041,22 @@
       <c r="F229" t="inlineStr"/>
       <c r="G229" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1988</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>300726064012887</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -15071,7 +15071,7 @@
       </c>
       <c r="M229" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N229" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>300726064012731</t>
+          <t>300726064012903</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>300726064012590</t>
+          <t>300726064012106</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -15248,7 +15248,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>300726064012700</t>
+          <t>300726064012606</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15312,7 +15312,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>300726064011668</t>
+          <t>300726064012950</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15376,7 +15376,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>300726064011950</t>
+          <t>300726064012528</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>300726064012903</t>
+          <t>300726064013028</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15504,7 +15504,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>300726064012106</t>
+          <t>300726064013012</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -15568,7 +15568,7 @@
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>300726064012606</t>
+          <t>300726064012965</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15632,7 +15632,7 @@
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>300726064012950</t>
+          <t>300726064011856</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -15696,7 +15696,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>300726064012825</t>
+          <t>300726064012840</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -15760,7 +15760,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>300726064013012</t>
+          <t>300726064012122</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -15824,7 +15824,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>300726064012622</t>
+          <t>300726064011872</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -15888,7 +15888,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>300726064012934</t>
+          <t>300726064011934</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -15952,7 +15952,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>300726064011856</t>
+          <t>300726064012997</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -16016,7 +16016,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>300726064012840</t>
+          <t>300726064012856</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16080,7 +16080,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>300726064012122</t>
+          <t>300726064012090</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -16112,7 +16112,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C246" t="inlineStr"/>
@@ -16129,22 +16129,22 @@
       <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>1988</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>300726064011872</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -16159,7 +16159,7 @@
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N246" t="inlineStr">
@@ -16208,7 +16208,7 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>300726064012559</t>
+          <t>300726064011668</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -16272,7 +16272,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>300726064012715</t>
+          <t>300726064012872</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>300726064012872</t>
+          <t>300726064012715</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>300726064012997</t>
+          <t>300726064012825</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -16464,7 +16464,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>300726064012856</t>
+          <t>300726064012559</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -16528,7 +16528,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>300726064012090</t>
+          <t>300726064012934</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -16560,7 +16560,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C253" t="inlineStr"/>
@@ -16577,22 +16577,22 @@
       <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1988</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>300726064012622</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -16607,7 +16607,7 @@
       </c>
       <c r="M253" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N253" t="inlineStr">
@@ -16641,22 +16641,22 @@
       <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>180226073056680</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -16671,7 +16671,7 @@
       </c>
       <c r="M254" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N254" t="inlineStr">
@@ -16705,22 +16705,22 @@
       <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056680</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>19</t>
         </is>
       </c>
       <c r="N255" t="inlineStr">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>280726145222572</t>
+          <t>280726145222650</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -16912,7 +16912,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>280726145222650</t>
+          <t>280726145222509</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -16976,7 +16976,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>280726145222509</t>
+          <t>280726145222572</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 11/08/2026 07:53:30
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 11/08/2026 13:45:08
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 11/08/2026 19:19:25
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -683,12 +683,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -705,22 +705,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1974</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1974</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -907,12 +907,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1003,12 +1003,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1974</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1089,22 +1089,22 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1195,12 +1195,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -1217,22 +1217,22 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1974</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1803,12 +1803,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2507,12 +2507,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2571,12 +2571,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>210726125342857</t>
+          <t>210726125342716</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>24</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>210726125342810</t>
+          <t>210726125342888</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>210726125342779</t>
+          <t>210726125342810</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>210726125342888</t>
+          <t>210726125342825</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>210726125342872</t>
+          <t>210726125342779</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2891,12 +2891,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>210726125342716</t>
+          <t>210726125342763</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>210726125342763</t>
+          <t>210726125342857</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>210726125342825</t>
+          <t>210726125342872</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3201,22 +3201,22 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3393,22 +3393,22 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3467,12 +3467,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3563,12 +3563,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CAL-027-001-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -3585,27 +3585,27 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132439966</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3627,12 +3627,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132440497</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3777,22 +3777,22 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3905,22 +3905,22 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3969,22 +3969,22 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4011,12 +4011,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4097,22 +4097,22 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4139,12 +4139,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>110226132440497</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4267,12 +4267,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-001-002</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
@@ -4289,27 +4289,27 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132439966</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4528,7 +4528,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132439700</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4737,22 +4737,22 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4865,22 +4865,22 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4929,22 +4929,22 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5163,12 +5163,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439700</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5249,22 +5249,22 @@
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5279,7 +5279,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5441,22 +5441,22 @@
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5505,22 +5505,22 @@
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -5953,27 +5953,27 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6017,27 +6017,27 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6145,12 +6145,12 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6273,12 +6273,12 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6475,12 +6475,12 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6495,7 +6495,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6593,12 +6593,12 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,12 +6913,12 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7563,12 +7563,12 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7617,22 +7617,22 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7681,12 +7681,12 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7809,12 +7809,12 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7883,12 +7883,12 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8171,12 +8171,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8363,12 +8363,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
@@ -8395,12 +8395,12 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8459,12 +8459,12 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8555,12 +8555,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C128" t="inlineStr"/>
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8833,22 +8833,22 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9003,12 +9003,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
@@ -9025,22 +9025,22 @@
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9707,12 +9707,12 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C146" t="inlineStr"/>
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -10123,12 +10123,12 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -10256,7 +10256,7 @@
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -10315,12 +10315,12 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -10561,22 +10561,22 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>19/11/2031</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1958</t>
+          <t>1926</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226062756227</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10591,7 +10591,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N159" t="inlineStr">
@@ -10625,22 +10625,22 @@
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>19/11/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1926</t>
+          <t>1958</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>200226062756227</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10655,7 +10655,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
@@ -10768,7 +10768,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>200226070819709</t>
+          <t>200226062756258</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>200226062756258</t>
+          <t>200226070819709</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -11009,12 +11009,12 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050826061104264</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11201,12 +11201,12 @@
       <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>050526131349498</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>050826061104264</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11531,12 +11531,12 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -11713,22 +11713,22 @@
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11792,7 +11792,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11824,7 +11824,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
@@ -11841,22 +11841,22 @@
       <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050526131349498</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -12043,12 +12043,12 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12144,7 +12144,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
@@ -12161,22 +12161,22 @@
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12208,7 +12208,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12673,22 +12673,22 @@
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -12737,22 +12737,22 @@
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12875,12 +12875,12 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -13003,12 +13003,12 @@
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13023,7 +13023,7 @@
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N197" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>300726064012668</t>
+          <t>300726064011997</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>300726064012684</t>
+          <t>300726064011981</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>300726064012918</t>
+          <t>300726064012012</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13424,7 +13424,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C204" t="inlineStr"/>
@@ -13441,22 +13441,22 @@
       <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1988</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>300726064012637</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13471,7 +13471,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N204" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>300726064012512</t>
+          <t>300726064012590</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>300726064011997</t>
+          <t>300726064012637</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>300726064013043</t>
+          <t>300726064011903</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>300726064011965</t>
+          <t>300726064012512</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>300726064011653</t>
+          <t>300726064012700</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>300726064012575</t>
+          <t>300726064011950</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>300726064011903</t>
+          <t>300726064012903</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>300726064011981</t>
+          <t>300726064012684</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>300726064011887</t>
+          <t>300726064012106</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14064,7 +14064,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C214" t="inlineStr"/>
@@ -14081,12 +14081,12 @@
       <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1988</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>300726064013012</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>300726064012028</t>
+          <t>300726064012856</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>300726064012981</t>
+          <t>300726064012668</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>300726064012543</t>
+          <t>300726064012575</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -14320,7 +14320,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C218" t="inlineStr"/>
@@ -14337,12 +14337,12 @@
       <c r="F218" t="inlineStr"/>
       <c r="G218" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>1988</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>300726064012793</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -14416,7 +14416,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>300726064011918</t>
+          <t>300726064012981</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>300726064012012</t>
+          <t>300726064012090</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>300726064012809</t>
+          <t>300726064012543</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -14576,7 +14576,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C222" t="inlineStr"/>
@@ -14593,22 +14593,22 @@
       <c r="F222" t="inlineStr"/>
       <c r="G222" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1988</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>300726064011918</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -14623,7 +14623,7 @@
       </c>
       <c r="M222" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N222" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>300726064012731</t>
+          <t>300726064012872</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>300726064012590</t>
+          <t>300726064012559</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>300726064012700</t>
+          <t>300726064012731</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>300726064012653</t>
+          <t>300726064011934</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14928,7 +14928,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>300726064011950</t>
+          <t>300726064012887</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -14992,7 +14992,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>300726064012497</t>
+          <t>300726064012653</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>300726064012887</t>
+          <t>300726064012809</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>300726064012903</t>
+          <t>300726064011887</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>300726064012106</t>
+          <t>300726064013043</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -15248,7 +15248,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>300726064012606</t>
+          <t>300726064012028</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15312,7 +15312,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>300726064012950</t>
+          <t>300726064012793</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15376,7 +15376,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>300726064012528</t>
+          <t>300726064011965</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>300726064013028</t>
+          <t>300726064012606</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15504,7 +15504,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>300726064013012</t>
+          <t>300726064012950</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -15568,7 +15568,7 @@
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>300726064012965</t>
+          <t>300726064012918</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15632,7 +15632,7 @@
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>300726064011856</t>
+          <t>300726064011653</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -15696,7 +15696,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>300726064012840</t>
+          <t>300726064011856</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -15760,7 +15760,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>300726064012122</t>
+          <t>300726064012840</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -15824,7 +15824,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>300726064011872</t>
+          <t>300726064012122</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -15888,7 +15888,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>300726064011934</t>
+          <t>300726064011872</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -15952,7 +15952,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>300726064012997</t>
+          <t>300726064012497</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -16016,7 +16016,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>300726064012856</t>
+          <t>300726064012528</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16080,7 +16080,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>300726064012090</t>
+          <t>300726064013028</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -16112,7 +16112,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C246" t="inlineStr"/>
@@ -16129,22 +16129,22 @@
       <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1988</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>300726064012965</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -16159,7 +16159,7 @@
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N246" t="inlineStr">
@@ -16272,7 +16272,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>300726064012872</t>
+          <t>300726064012997</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>300726064012715</t>
+          <t>300726064012825</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -16368,7 +16368,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C250" t="inlineStr"/>
@@ -16385,22 +16385,22 @@
       <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>1988</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>300726064012825</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -16415,7 +16415,7 @@
       </c>
       <c r="M250" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N250" t="inlineStr">
@@ -16464,7 +16464,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>300726064012559</t>
+          <t>300726064012622</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>300726064012622</t>
+          <t>300726064012715</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -16784,7 +16784,7 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222509</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>280726145222650</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -16912,7 +16912,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>280726145222509</t>
+          <t>280726145222650</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 12/08/2026 06:54:16
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -11009,12 +11009,12 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11073,12 +11073,12 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 12/08/2026 10:53:05
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -683,12 +683,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -705,22 +705,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1973</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1973</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -875,12 +875,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -976,7 +976,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1003,12 +1003,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1973</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1099,12 +1099,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1195,12 +1195,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -1217,22 +1217,22 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1973</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1803,12 +1803,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2379,12 +2379,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2731,12 +2731,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2753,22 +2753,22 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2817,22 +2817,22 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2859,12 +2859,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>110226132440497</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2923,12 +2923,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-001-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2960,12 +2960,12 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>110226132439966</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3051,12 +3051,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>110226132439700</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3115,12 +3115,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>110226132440497</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3179,12 +3179,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CAL-027-001-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -3216,12 +3216,12 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132439966</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3275,12 +3275,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132440513</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3457,22 +3457,22 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3627,12 +3627,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3659,12 +3659,12 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132440513</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3905,22 +3905,22 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3969,22 +3969,22 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4033,22 +4033,22 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4097,22 +4097,22 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4235,12 +4235,12 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4331,12 +4331,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132439700</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4481,22 +4481,22 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4673,22 +4673,22 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4865,22 +4865,22 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5697,12 +5697,12 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5889,12 +5889,12 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5963,12 +5963,12 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6017,12 +6017,12 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,12 +6081,12 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6145,22 +6145,22 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6529,12 +6529,12 @@
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6603,12 +6603,12 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6785,12 +6785,12 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6987,12 +6987,12 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7169,12 +7169,12 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,12 +7233,12 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7531,12 +7531,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C112" t="inlineStr"/>
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7659,12 +7659,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7723,12 +7723,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C115" t="inlineStr"/>
@@ -7755,12 +7755,12 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7775,7 +7775,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -7787,12 +7787,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7947,12 +7947,12 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8385,22 +8385,22 @@
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9259,12 +9259,12 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C139" t="inlineStr"/>
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9409,22 +9409,22 @@
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9611,12 +9611,12 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9739,12 +9739,12 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -10369,12 +10369,12 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10384,7 +10384,7 @@
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10416,7 +10416,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C157" t="inlineStr"/>
@@ -10433,22 +10433,22 @@
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10640,7 +10640,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -10689,22 +10689,22 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -10768,7 +10768,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>050526131349498</t>
+          <t>050826061104264</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10800,7 +10800,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C163" t="inlineStr"/>
@@ -10817,22 +10817,22 @@
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>050526131349498</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11120,7 +11120,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C168" t="inlineStr"/>
@@ -11137,22 +11137,22 @@
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050826061104264</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>200226062905996</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226062905996</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
@@ -11585,22 +11585,22 @@
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -11713,22 +11713,22 @@
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11851,12 +11851,12 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -11915,12 +11915,12 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -12043,12 +12043,12 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12107,12 +12107,12 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12161,22 +12161,22 @@
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1957</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12427,12 +12427,12 @@
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12481,22 +12481,22 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1957</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12555,12 +12555,12 @@
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12619,12 +12619,12 @@
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>44</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>44</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12752,7 +12752,7 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>300726064012559</t>
+          <t>300726064012731</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12816,7 +12816,7 @@
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>300726064012637</t>
+          <t>300726064011856</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12880,7 +12880,7 @@
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>300726064012512</t>
+          <t>300726064011918</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12944,7 +12944,7 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>300726064011934</t>
+          <t>300726064012575</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -13008,7 +13008,7 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>300726064011997</t>
+          <t>300726064012981</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13072,7 +13072,7 @@
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>300726064012887</t>
+          <t>300726064012825</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -13104,7 +13104,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
@@ -13121,12 +13121,12 @@
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13136,7 +13136,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>300726064012653</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13168,7 +13168,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
@@ -13185,12 +13185,12 @@
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1987</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>300726064011950</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>300726064011903</t>
+          <t>300726064012512</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>300726064012872</t>
+          <t>300726064012637</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>300726064012543</t>
+          <t>300726064012903</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>300726064012090</t>
+          <t>300726064011887</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>300726064012856</t>
+          <t>300726064011668</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>300726064013012</t>
+          <t>300726064011997</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>300726064012106</t>
+          <t>300726064011903</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>300726064011856</t>
+          <t>300726064012543</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>300726064012700</t>
+          <t>300726064012684</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>300726064012590</t>
+          <t>300726064012668</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>300726064012825</t>
+          <t>300726064011981</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>300726064011668</t>
+          <t>300726064012012</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>300726064012012</t>
+          <t>300726064012590</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>300726064011981</t>
+          <t>300726064012700</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>300726064011887</t>
+          <t>300726064013012</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>300726064012684</t>
+          <t>300726064012106</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>300726064012668</t>
+          <t>300726064012856</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -14416,7 +14416,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>300726064012903</t>
+          <t>300726064012090</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>300726064011950</t>
+          <t>300726064012872</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>300726064012575</t>
+          <t>300726064012559</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -14608,7 +14608,7 @@
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>300726064011918</t>
+          <t>300726064012887</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>300726064012840</t>
+          <t>300726064011934</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>300726064012122</t>
+          <t>300726064012653</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>300726064011872</t>
+          <t>300726064012809</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>300726064012528</t>
+          <t>300726064013043</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14928,7 +14928,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>300726064012497</t>
+          <t>300726064012028</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -14992,7 +14992,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>300726064012997</t>
+          <t>300726064012793</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>300726064012950</t>
+          <t>300726064011965</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>300726064012606</t>
+          <t>300726064012918</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>300726064013028</t>
+          <t>300726064011653</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C232" t="inlineStr"/>
@@ -15233,22 +15233,22 @@
       <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1987</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>300726064012497</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15263,7 +15263,7 @@
       </c>
       <c r="M232" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N232" t="inlineStr">
@@ -15312,7 +15312,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>300726064012965</t>
+          <t>300726064012528</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15376,7 +15376,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>300726064011653</t>
+          <t>300726064013028</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>300726064012918</t>
+          <t>300726064012965</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15504,7 +15504,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>300726064012715</t>
+          <t>300726064012622</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -15568,7 +15568,7 @@
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>300726064011965</t>
+          <t>300726064012934</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15632,7 +15632,7 @@
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>300726064012793</t>
+          <t>300726064012606</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -15696,7 +15696,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>300726064012731</t>
+          <t>300726064012715</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -15760,7 +15760,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>300726064012028</t>
+          <t>300726064012950</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -15792,7 +15792,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C241" t="inlineStr"/>
@@ -15809,22 +15809,22 @@
       <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>300726064013043</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -15839,7 +15839,7 @@
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N241" t="inlineStr">
@@ -15888,7 +15888,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>300726064012934</t>
+          <t>300726064012997</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -15952,7 +15952,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>300726064012622</t>
+          <t>300726064012122</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -16016,7 +16016,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>300726064012981</t>
+          <t>300726064011872</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16080,7 +16080,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>300726064012809</t>
+          <t>300726064012840</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -16272,7 +16272,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>280726145222697</t>
+          <t>280726145222478</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>280726145222509</t>
+          <t>280726145222603</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>280726145222603</t>
+          <t>280726145222665</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -16464,7 +16464,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -16523,12 +16523,12 @@
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>280726145222353</t>
+          <t>280726145222290</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -16543,7 +16543,7 @@
       </c>
       <c r="M252" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N252" t="inlineStr">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>280726145222150</t>
+          <t>280726145222509</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -16656,7 +16656,7 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>280726145222228</t>
+          <t>280726145222634</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -16688,7 +16688,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C255" t="inlineStr"/>
@@ -16705,22 +16705,22 @@
       <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280726145222415</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N255" t="inlineStr">
@@ -16784,7 +16784,7 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>280726145222478</t>
+          <t>280726145222134</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>280726145222447</t>
+          <t>280726145222197</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -16880,7 +16880,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C258" t="inlineStr"/>
@@ -16897,22 +16897,22 @@
       <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>280726145222181</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -16927,7 +16927,7 @@
       </c>
       <c r="M258" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N258" t="inlineStr">
@@ -16976,7 +16976,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>280726145221681</t>
+          <t>280726145222009</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>280726145222103</t>
+          <t>280726145221994</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -17072,7 +17072,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C261" t="inlineStr"/>
@@ -17089,22 +17089,22 @@
       <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -17119,7 +17119,7 @@
       </c>
       <c r="M261" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N261" t="inlineStr">
@@ -17168,7 +17168,7 @@
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>280726145222572</t>
+          <t>280726145222681</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
@@ -17232,7 +17232,7 @@
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>280726145222119</t>
+          <t>280726145221697</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -17296,7 +17296,7 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>280726145222415</t>
+          <t>280726145222572</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -17360,7 +17360,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>280726145222634</t>
+          <t>280726145222119</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -17424,7 +17424,7 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>280726145222134</t>
+          <t>280726145222587</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -17488,7 +17488,7 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>280726145222650</t>
+          <t>280726145222212</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222525</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -17616,7 +17616,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>280726145222681</t>
+          <t>280726145222244</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -17680,7 +17680,7 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>280726145222197</t>
+          <t>280726145222322</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -17744,7 +17744,7 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>280726145222181</t>
+          <t>280726145222650</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>280726145221994</t>
+          <t>280726145222103</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -17872,7 +17872,7 @@
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>280726145222540</t>
+          <t>280726145221681</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -17936,7 +17936,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>280726145222165</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -17968,7 +17968,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C275" t="inlineStr"/>
@@ -17985,22 +17985,22 @@
       <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>280726145222009</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -18015,7 +18015,7 @@
       </c>
       <c r="M275" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N275" t="inlineStr">
@@ -18032,7 +18032,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C276" t="inlineStr"/>
@@ -18049,22 +18049,22 @@
       <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>280726145222337</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -18079,7 +18079,7 @@
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N276" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>280726145222494</t>
+          <t>280726145222447</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -18192,7 +18192,7 @@
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>280726145221697</t>
+          <t>280726145222556</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
@@ -18251,12 +18251,12 @@
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>280726145222290</t>
+          <t>280726145222165</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
@@ -18271,7 +18271,7 @@
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N279" t="inlineStr">
@@ -18320,7 +18320,7 @@
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>280726145222556</t>
+          <t>280726145222540</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
@@ -18384,7 +18384,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>280726145222337</t>
+          <t>280726145222494</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -18448,7 +18448,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>280726145222665</t>
+          <t>280726145222150</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -18512,7 +18512,7 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>280726145222619</t>
+          <t>280726145222353</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -18576,7 +18576,7 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -18640,7 +18640,7 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>280726145222587</t>
+          <t>280726145222697</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -18704,7 +18704,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>280726145222525</t>
+          <t>280726145222228</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -18736,7 +18736,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C287" t="inlineStr"/>
@@ -18753,22 +18753,22 @@
       <c r="F287" t="inlineStr"/>
       <c r="G287" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>280726145222322</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
@@ -18783,7 +18783,7 @@
       </c>
       <c r="M287" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N287" t="inlineStr">
@@ -18832,7 +18832,7 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>280726145222244</t>
+          <t>280726145222619</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -18864,7 +18864,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C289" t="inlineStr"/>
@@ -18881,22 +18881,22 @@
       <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>280726145222212</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -18911,7 +18911,7 @@
       </c>
       <c r="M289" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N289" t="inlineStr">
@@ -18960,7 +18960,7 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>280726145222431</t>
+          <t>280726145222306</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -19056,7 +19056,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C292" t="inlineStr"/>
@@ -19073,22 +19073,22 @@
       <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J292" t="inlineStr">
         <is>
-          <t>280726145222400</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
@@ -19103,7 +19103,7 @@
       </c>
       <c r="M292" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N292" t="inlineStr">
@@ -19120,7 +19120,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C293" t="inlineStr"/>
@@ -19137,22 +19137,22 @@
       <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J293" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>280726145222400</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
@@ -19167,7 +19167,7 @@
       </c>
       <c r="M293" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N293" t="inlineStr">
@@ -19216,7 +19216,7 @@
       </c>
       <c r="J294" t="inlineStr">
         <is>
-          <t>280726145222259</t>
+          <t>280726145222431</t>
         </is>
       </c>
       <c r="K294" t="inlineStr">
@@ -19248,7 +19248,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C295" t="inlineStr"/>
@@ -19265,22 +19265,22 @@
       <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>280726145222259</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
@@ -19295,7 +19295,7 @@
       </c>
       <c r="M295" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N295" t="inlineStr">
@@ -19312,7 +19312,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C296" t="inlineStr"/>
@@ -19329,22 +19329,22 @@
       <c r="F296" t="inlineStr"/>
       <c r="G296" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>280726145222306</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
@@ -19359,7 +19359,7 @@
       </c>
       <c r="M296" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N296" t="inlineStr">
@@ -19440,7 +19440,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C298" t="inlineStr"/>
@@ -19457,27 +19457,27 @@
       <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr">
         <is>
-          <t>09/12/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>77</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>180626072347907</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L298" t="inlineStr">
@@ -19487,7 +19487,7 @@
       </c>
       <c r="M298" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>77</t>
         </is>
       </c>
       <c r="N298" t="inlineStr">
@@ -19504,7 +19504,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C299" t="inlineStr"/>
@@ -19521,27 +19521,27 @@
       <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>09/12/2031</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1945</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>110226132440294</t>
+          <t>180626072347907</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L299" t="inlineStr">
@@ -19551,7 +19551,7 @@
       </c>
       <c r="M299" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>50</t>
         </is>
       </c>
       <c r="N299" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 12/08/2026 11:05:36
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -683,12 +683,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -705,22 +705,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1973</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -875,12 +875,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,12 +897,12 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1973</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1099,12 +1099,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1973</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1195,12 +1195,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -1217,22 +1217,22 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1973</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1803,12 +1803,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1995,12 +1995,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2379,12 +2379,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2731,12 +2731,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2827,12 +2827,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2923,12 +2923,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-001-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2945,27 +2945,27 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>110226132439966</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3051,12 +3051,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-001-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3088,12 +3088,12 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>110226132439966</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3211,12 +3211,12 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3393,12 +3393,12 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132440513</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3435,12 +3435,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3499,12 +3499,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132439700</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3649,12 +3649,12 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132440513</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3777,22 +3777,22 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3905,22 +3905,22 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4107,12 +4107,12 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4289,22 +4289,22 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4331,12 +4331,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132439700</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4417,22 +4417,22 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,22 +4609,22 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4737,22 +4737,22 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4865,22 +4865,22 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4929,22 +4929,22 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -5003,12 +5003,12 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5441,27 +5441,27 @@
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5505,27 +5505,27 @@
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -5633,22 +5633,22 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5761,12 +5761,12 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5889,12 +5889,12 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5953,22 +5953,22 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6017,12 +6017,12 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6145,12 +6145,12 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6401,12 +6401,12 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6529,22 +6529,22 @@
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6559,7 +6559,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -6593,12 +6593,12 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6657,12 +6657,12 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,12 +6913,12 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6987,12 +6987,12 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7297,12 +7297,12 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7403,12 +7403,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C110" t="inlineStr"/>
@@ -7435,12 +7435,12 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7531,12 +7531,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C112" t="inlineStr"/>
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7787,12 +7787,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7851,12 +7851,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7947,12 +7947,12 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8385,22 +8385,22 @@
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8939,12 +8939,12 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C134" t="inlineStr"/>
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9025,22 +9025,22 @@
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9259,12 +9259,12 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C139" t="inlineStr"/>
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9611,12 +9611,12 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9803,12 +9803,12 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N147" t="inlineStr">
@@ -10384,7 +10384,7 @@
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10416,7 +10416,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C157" t="inlineStr"/>
@@ -10433,22 +10433,22 @@
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050826061104264</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10561,12 +10561,12 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10640,7 +10640,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10689,12 +10689,12 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10704,7 +10704,7 @@
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
@@ -10753,22 +10753,22 @@
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>050826061104264</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -10800,7 +10800,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C163" t="inlineStr"/>
@@ -10817,22 +10817,22 @@
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
@@ -10864,7 +10864,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C164" t="inlineStr"/>
@@ -10881,22 +10881,22 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>050526131349498</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11120,7 +11120,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C168" t="inlineStr"/>
@@ -11137,22 +11137,22 @@
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11184,7 +11184,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C169" t="inlineStr"/>
@@ -11201,22 +11201,22 @@
       <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>050526131349498</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11344,7 +11344,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
@@ -11585,22 +11585,22 @@
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -11659,12 +11659,12 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -11713,22 +11713,22 @@
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11777,22 +11777,22 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11824,7 +11824,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
@@ -11841,22 +11841,22 @@
       <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -12161,22 +12161,22 @@
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1957</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12363,12 +12363,12 @@
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1957</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12491,12 +12491,12 @@
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12752,7 +12752,7 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>300726064012731</t>
+          <t>300726064012528</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12816,7 +12816,7 @@
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>300726064011856</t>
+          <t>300726064012497</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12880,7 +12880,7 @@
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>300726064011918</t>
+          <t>300726064012512</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12944,7 +12944,7 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>300726064012575</t>
+          <t>300726064012637</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -13008,7 +13008,7 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>300726064012981</t>
+          <t>300726064011653</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13072,7 +13072,7 @@
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>300726064012825</t>
+          <t>300726064011997</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -13104,7 +13104,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
@@ -13121,12 +13121,12 @@
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1987</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13136,7 +13136,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>300726064012918</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>300726064011950</t>
+          <t>300726064011903</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>300726064012512</t>
+          <t>300726064011965</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>300726064012637</t>
+          <t>300726064012793</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>300726064012903</t>
+          <t>300726064012543</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>300726064011887</t>
+          <t>300726064012028</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>300726064011668</t>
+          <t>300726064013043</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>300726064011997</t>
+          <t>300726064012809</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>300726064011903</t>
+          <t>300726064012653</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>300726064012543</t>
+          <t>300726064012887</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>300726064012684</t>
+          <t>300726064011934</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>300726064012668</t>
+          <t>300726064011856</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>300726064011981</t>
+          <t>300726064012559</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>300726064012012</t>
+          <t>300726064012872</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14000,7 +14000,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C213" t="inlineStr"/>
@@ -14017,22 +14017,22 @@
       <c r="F213" t="inlineStr"/>
       <c r="G213" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1987</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>300726064012090</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14047,7 +14047,7 @@
       </c>
       <c r="M213" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N213" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>300726064012590</t>
+          <t>300726064012856</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>300726064012700</t>
+          <t>300726064013012</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>300726064013012</t>
+          <t>300726064012106</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>300726064012106</t>
+          <t>300726064012825</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>300726064012856</t>
+          <t>300726064011668</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -14416,7 +14416,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>300726064012090</t>
+          <t>300726064012700</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>300726064012872</t>
+          <t>300726064012590</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>300726064012559</t>
+          <t>300726064011887</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -14576,7 +14576,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C222" t="inlineStr"/>
@@ -14593,22 +14593,22 @@
       <c r="F222" t="inlineStr"/>
       <c r="G222" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>300726064012887</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -14623,7 +14623,7 @@
       </c>
       <c r="M222" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N222" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>300726064011934</t>
+          <t>300726064012012</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>300726064012653</t>
+          <t>300726064011981</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>300726064012809</t>
+          <t>300726064012903</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>300726064013043</t>
+          <t>300726064012684</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14928,7 +14928,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>300726064012028</t>
+          <t>300726064012668</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -14992,7 +14992,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>300726064012793</t>
+          <t>300726064011950</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>300726064011965</t>
+          <t>300726064012575</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>300726064012918</t>
+          <t>300726064011918</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>300726064011653</t>
+          <t>300726064013028</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -15248,7 +15248,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>300726064012497</t>
+          <t>300726064012965</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15312,7 +15312,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>300726064012528</t>
+          <t>300726064012840</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15376,7 +15376,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>300726064013028</t>
+          <t>300726064012122</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>300726064012965</t>
+          <t>300726064011872</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15504,7 +15504,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>300726064012622</t>
+          <t>300726064012950</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -15568,7 +15568,7 @@
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>300726064012934</t>
+          <t>300726064012606</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15600,7 +15600,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C238" t="inlineStr"/>
@@ -15617,12 +15617,12 @@
       <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -15632,7 +15632,7 @@
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>300726064012606</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -15696,7 +15696,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>300726064012715</t>
+          <t>300726064012981</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -15760,7 +15760,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>300726064012950</t>
+          <t>300726064012622</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -15792,7 +15792,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C241" t="inlineStr"/>
@@ -15809,22 +15809,22 @@
       <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1987</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>300726064012934</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -15839,7 +15839,7 @@
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N241" t="inlineStr">
@@ -15888,7 +15888,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>300726064012997</t>
+          <t>300726064012715</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -15952,7 +15952,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>300726064012122</t>
+          <t>300726064012731</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -16016,7 +16016,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>300726064011872</t>
+          <t>300726064012997</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16048,7 +16048,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C245" t="inlineStr"/>
@@ -16065,22 +16065,22 @@
       <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>300726064012840</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -16095,7 +16095,7 @@
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N245" t="inlineStr">
@@ -16272,7 +16272,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>280726145222478</t>
+          <t>280726145222681</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>280726145222603</t>
+          <t>280726145221994</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>280726145222665</t>
+          <t>280726145222478</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -16464,7 +16464,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222603</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -16523,12 +16523,12 @@
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>280726145222290</t>
+          <t>280726145222009</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -16543,7 +16543,7 @@
       </c>
       <c r="M252" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N252" t="inlineStr">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>280726145222509</t>
+          <t>280726145222119</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -16656,7 +16656,7 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>280726145222634</t>
+          <t>280726145222509</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -16720,7 +16720,7 @@
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>280726145222415</t>
+          <t>280726145222103</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -16779,12 +16779,12 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>280726145222134</t>
+          <t>280726145222290</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -16799,7 +16799,7 @@
       </c>
       <c r="M256" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N256" t="inlineStr">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>280726145222197</t>
+          <t>280726145221681</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -16912,7 +16912,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>280726145222181</t>
+          <t>280726145222415</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -16976,7 +16976,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>280726145222009</t>
+          <t>280726145222634</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>280726145221994</t>
+          <t>280726145222134</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -17072,7 +17072,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C261" t="inlineStr"/>
@@ -17089,22 +17089,22 @@
       <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>280726145222197</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -17119,7 +17119,7 @@
       </c>
       <c r="M261" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N261" t="inlineStr">
@@ -17168,7 +17168,7 @@
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>280726145222681</t>
+          <t>280726145222181</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
@@ -17200,7 +17200,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C263" t="inlineStr"/>
@@ -17217,22 +17217,22 @@
       <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>280726145221697</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -17247,7 +17247,7 @@
       </c>
       <c r="M263" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N263" t="inlineStr">
@@ -17360,7 +17360,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>280726145222119</t>
+          <t>280726145222665</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -17424,7 +17424,7 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>280726145222587</t>
+          <t>280726145222447</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -17456,7 +17456,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C267" t="inlineStr"/>
@@ -17473,22 +17473,22 @@
       <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1827</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>280726145222212</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -17503,7 +17503,7 @@
       </c>
       <c r="M267" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N267" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>280726145222525</t>
+          <t>280726145221697</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -17616,7 +17616,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>280726145222244</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -17680,7 +17680,7 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>280726145222322</t>
+          <t>280726145222650</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -17744,7 +17744,7 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>280726145222650</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>280726145222103</t>
+          <t>280726145222587</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -17872,7 +17872,7 @@
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>280726145221681</t>
+          <t>280726145222525</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -17936,7 +17936,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222322</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -18032,7 +18032,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C276" t="inlineStr"/>
@@ -18049,22 +18049,22 @@
       <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>280726145222337</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -18079,7 +18079,7 @@
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N276" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>280726145222447</t>
+          <t>280726145222494</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -18192,7 +18192,7 @@
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>280726145222556</t>
+          <t>280726145222228</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
@@ -18256,7 +18256,7 @@
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>280726145222165</t>
+          <t>280726145222337</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
@@ -18320,7 +18320,7 @@
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>280726145222540</t>
+          <t>280726145222697</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
@@ -18384,7 +18384,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>280726145222494</t>
+          <t>280726145222212</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -18448,7 +18448,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>280726145222150</t>
+          <t>280726145222556</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -18512,7 +18512,7 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>280726145222353</t>
+          <t>280726145222244</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -18576,7 +18576,7 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>280726145222619</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -18640,7 +18640,7 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>280726145222697</t>
+          <t>280726145222165</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -18704,7 +18704,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>280726145222228</t>
+          <t>280726145222540</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -18736,7 +18736,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C287" t="inlineStr"/>
@@ -18753,22 +18753,22 @@
       <c r="F287" t="inlineStr"/>
       <c r="G287" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
@@ -18783,7 +18783,7 @@
       </c>
       <c r="M287" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N287" t="inlineStr">
@@ -18832,7 +18832,7 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>280726145222619</t>
+          <t>280726145222353</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -18864,7 +18864,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C289" t="inlineStr"/>
@@ -18881,22 +18881,22 @@
       <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280726145222150</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -18911,7 +18911,7 @@
       </c>
       <c r="M289" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N289" t="inlineStr">
@@ -18960,7 +18960,7 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>280726145222306</t>
+          <t>280726145222259</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -19019,12 +19019,12 @@
       </c>
       <c r="I291" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J291" t="inlineStr">
         <is>
-          <t>280726145222384</t>
+          <t>280726145222400</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
@@ -19039,7 +19039,7 @@
       </c>
       <c r="M291" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N291" t="inlineStr">
@@ -19152,7 +19152,7 @@
       </c>
       <c r="J293" t="inlineStr">
         <is>
-          <t>280726145222400</t>
+          <t>280726145222306</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
@@ -19248,7 +19248,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C295" t="inlineStr"/>
@@ -19265,22 +19265,22 @@
       <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>280726145222259</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
@@ -19295,7 +19295,7 @@
       </c>
       <c r="M295" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N295" t="inlineStr">
@@ -19312,7 +19312,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C296" t="inlineStr"/>
@@ -19329,22 +19329,22 @@
       <c r="F296" t="inlineStr"/>
       <c r="G296" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>33</t>
         </is>
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>280726145222384</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
@@ -19359,7 +19359,7 @@
       </c>
       <c r="M296" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>33</t>
         </is>
       </c>
       <c r="N296" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 13/08/2026 06:02:21
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1916</t>
+          <t>1915</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1973</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1973</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1973</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1973</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1881</t>
+          <t>1880</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1811</t>
+          <t>1810</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1811</t>
+          <t>1810</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1879</t>
+          <t>1878</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1925</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1957</t>
+          <t>1956</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1925</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1957</t>
+          <t>1956</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -13446,7 +13446,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -13766,7 +13766,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -14086,7 +14086,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -14150,7 +14150,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -14214,7 +14214,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -14278,7 +14278,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -14406,7 +14406,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -14534,7 +14534,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -14598,7 +14598,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
@@ -14662,7 +14662,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -14726,7 +14726,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -14790,7 +14790,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -14854,7 +14854,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -14918,7 +14918,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -15046,7 +15046,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -15110,7 +15110,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -15174,7 +15174,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
@@ -15238,7 +15238,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -15302,7 +15302,7 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
@@ -15430,7 +15430,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -15622,7 +15622,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -15686,7 +15686,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -15750,7 +15750,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -15814,7 +15814,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -15878,7 +15878,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -15942,7 +15942,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -16006,7 +16006,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
@@ -16070,7 +16070,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -16134,7 +16134,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
@@ -16198,7 +16198,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
@@ -16262,7 +16262,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -16326,7 +16326,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -16390,7 +16390,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -16582,7 +16582,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -16646,7 +16646,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -16774,7 +16774,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -16902,7 +16902,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -16966,7 +16966,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -17030,7 +17030,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -17094,7 +17094,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
@@ -17158,7 +17158,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -17222,7 +17222,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
@@ -17350,7 +17350,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -17414,7 +17414,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -17478,7 +17478,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -17542,7 +17542,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -17606,7 +17606,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -17670,7 +17670,7 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
@@ -17734,7 +17734,7 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
@@ -17798,7 +17798,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -17862,7 +17862,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -17926,7 +17926,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -17990,7 +17990,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
@@ -18054,7 +18054,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>1827</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -18118,7 +18118,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -18182,7 +18182,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -18246,7 +18246,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -18310,7 +18310,7 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
@@ -18374,7 +18374,7 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -18502,7 +18502,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -18566,7 +18566,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
@@ -18630,7 +18630,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
@@ -18758,7 +18758,7 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
@@ -18822,7 +18822,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
@@ -18886,7 +18886,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -18950,7 +18950,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
@@ -19014,7 +19014,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -19078,7 +19078,7 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
@@ -19142,7 +19142,7 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -19270,7 +19270,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -19334,7 +19334,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -19398,7 +19398,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -19462,7 +19462,7 @@
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>1944</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
@@ -19526,7 +19526,7 @@
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -19590,7 +19590,7 @@
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
@@ -19654,7 +19654,7 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 13/08/2026 06:14:53
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -784,7 +784,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -843,12 +843,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1035,12 +1035,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1089,22 +1089,22 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1227,12 +1227,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1547,12 +1547,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1867,12 +1867,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2763,12 +2763,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2817,22 +2817,22 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3051,12 +3051,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3073,22 +3073,22 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>110226132439700</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3115,12 +3115,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>110226132440497</t>
+          <t>110226132440513</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CAL-027-001-002</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -3216,12 +3216,12 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132439966</t>
+          <t>110226132440497</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3275,12 +3275,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132440513</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-001-002</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3393,27 +3393,27 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132439966</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3499,12 +3499,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3627,12 +3627,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3659,12 +3659,12 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3691,12 +3691,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132439700</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4225,22 +4225,22 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4481,22 +4481,22 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4673,22 +4673,22 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4737,22 +4737,22 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4865,22 +4865,22 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5441,27 +5441,27 @@
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5505,27 +5505,27 @@
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5707,12 +5707,12 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5953,12 +5953,12 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6017,12 +6017,12 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,12 +6081,12 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6145,22 +6145,22 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6209,12 +6209,12 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6273,12 +6273,12 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6593,22 +6593,22 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6785,12 +6785,12 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,12 +6913,12 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7115,12 +7115,12 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,12 +7233,12 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7297,12 +7297,12 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7361,12 +7361,12 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7403,12 +7403,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C110" t="inlineStr"/>
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7467,12 +7467,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C111" t="inlineStr"/>
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7531,12 +7531,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C112" t="inlineStr"/>
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7755,12 +7755,12 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7775,7 +7775,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -7787,12 +7787,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7915,12 +7915,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C118" t="inlineStr"/>
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8011,12 +8011,12 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -8043,12 +8043,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8321,22 +8321,22 @@
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8683,12 +8683,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C130" t="inlineStr"/>
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9409,22 +9409,22 @@
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -10049,22 +10049,22 @@
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
-          <t>19/11/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1956</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>200226062756227</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -10113,22 +10113,22 @@
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>19/11/2031</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1956</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226062756227</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -10369,12 +10369,12 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1993</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10384,7 +10384,7 @@
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>050826061104264</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>050526131349498</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10561,12 +10561,12 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
@@ -10625,22 +10625,22 @@
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10655,7 +10655,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -10689,22 +10689,22 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -10768,7 +10768,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>050526131349498</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10864,7 +10864,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C164" t="inlineStr"/>
@@ -10881,22 +10881,22 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050826061104264</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>200226062905996</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226062905996</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11585,22 +11585,22 @@
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11777,22 +11777,22 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11824,7 +11824,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
@@ -11841,22 +11841,22 @@
       <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -11915,12 +11915,12 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -12043,12 +12043,12 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12107,12 +12107,12 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12299,12 +12299,12 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12353,22 +12353,22 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1956</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12427,12 +12427,12 @@
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12481,22 +12481,22 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1956</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12555,12 +12555,12 @@
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12619,12 +12619,12 @@
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>44</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>44</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12752,7 +12752,7 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>300726064012559</t>
+          <t>300726064011918</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12816,7 +12816,7 @@
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>300726064012637</t>
+          <t>300726064012575</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12880,7 +12880,7 @@
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>300726064012512</t>
+          <t>300726064011950</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12944,7 +12944,7 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>300726064011934</t>
+          <t>300726064012668</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -13008,7 +13008,7 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>300726064011997</t>
+          <t>300726064012684</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13072,7 +13072,7 @@
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>300726064012887</t>
+          <t>300726064012903</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -13136,7 +13136,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>300726064012653</t>
+          <t>300726064011981</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13168,7 +13168,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
@@ -13185,12 +13185,12 @@
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>300726064012012</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13232,7 +13232,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C201" t="inlineStr"/>
@@ -13249,22 +13249,22 @@
       <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>300726064011903</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13279,7 +13279,7 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>300726064012872</t>
+          <t>300726064011887</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>300726064012543</t>
+          <t>300726064012590</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>300726064012090</t>
+          <t>300726064012700</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>300726064012856</t>
+          <t>300726064011668</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>300726064013012</t>
+          <t>300726064012825</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>300726064011856</t>
+          <t>300726064013012</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>300726064012700</t>
+          <t>300726064012856</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>300726064012590</t>
+          <t>300726064012090</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>300726064012825</t>
+          <t>300726064012872</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>300726064011668</t>
+          <t>300726064012559</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14000,7 +14000,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C213" t="inlineStr"/>
@@ -14017,22 +14017,22 @@
       <c r="F213" t="inlineStr"/>
       <c r="G213" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>300726064011856</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14047,7 +14047,7 @@
       </c>
       <c r="M213" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N213" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>300726064012012</t>
+          <t>300726064011934</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>300726064011981</t>
+          <t>300726064012887</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>300726064011887</t>
+          <t>300726064012653</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>300726064012684</t>
+          <t>300726064012809</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>300726064012668</t>
+          <t>300726064013043</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -14416,7 +14416,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>300726064012903</t>
+          <t>300726064012028</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>300726064011950</t>
+          <t>300726064012793</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>300726064012575</t>
+          <t>300726064012543</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -14608,7 +14608,7 @@
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>300726064011918</t>
+          <t>300726064011965</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>300726064012840</t>
+          <t>300726064011903</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>300726064012122</t>
+          <t>300726064012918</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>300726064011872</t>
+          <t>300726064011997</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>300726064012528</t>
+          <t>300726064011653</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14992,7 +14992,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>300726064012997</t>
+          <t>300726064012637</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>300726064012950</t>
+          <t>300726064012512</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>300726064012606</t>
+          <t>300726064012528</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C232" t="inlineStr"/>
@@ -15233,22 +15233,22 @@
       <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>300726064012965</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15263,7 +15263,7 @@
       </c>
       <c r="M232" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N232" t="inlineStr">
@@ -15312,7 +15312,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>300726064012965</t>
+          <t>300726064012840</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15376,7 +15376,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>300726064011653</t>
+          <t>300726064012950</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>300726064012918</t>
+          <t>300726064012606</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15504,7 +15504,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>300726064012715</t>
+          <t>300726064012122</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -15536,7 +15536,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C237" t="inlineStr"/>
@@ -15553,12 +15553,12 @@
       <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -15568,7 +15568,7 @@
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>300726064011965</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15632,7 +15632,7 @@
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>300726064012793</t>
+          <t>300726064011872</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -15696,7 +15696,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>300726064012731</t>
+          <t>300726064012981</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -15760,7 +15760,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>300726064012028</t>
+          <t>300726064012622</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -15824,7 +15824,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>300726064013043</t>
+          <t>300726064012934</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -15888,7 +15888,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>300726064012934</t>
+          <t>300726064012715</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -15952,7 +15952,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>300726064012622</t>
+          <t>300726064012997</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -16016,7 +16016,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>300726064012981</t>
+          <t>300726064012731</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16048,7 +16048,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C245" t="inlineStr"/>
@@ -16065,22 +16065,22 @@
       <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>300726064012809</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -16095,7 +16095,7 @@
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N245" t="inlineStr">
@@ -16272,7 +16272,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>280726145222697</t>
+          <t>280726145221994</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>280726145222509</t>
+          <t>280726145222681</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>280726145222603</t>
+          <t>280726145222478</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -16464,7 +16464,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>280726145222603</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -16528,7 +16528,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>280726145222353</t>
+          <t>280726145222009</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>280726145222150</t>
+          <t>280726145222509</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -16651,12 +16651,12 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>280726145222228</t>
+          <t>280726145222290</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -16671,7 +16671,7 @@
       </c>
       <c r="M254" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N254" t="inlineStr">
@@ -16688,7 +16688,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C255" t="inlineStr"/>
@@ -16705,22 +16705,22 @@
       <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280726145222119</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N255" t="inlineStr">
@@ -16784,7 +16784,7 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>280726145222478</t>
+          <t>280726145222103</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>280726145222447</t>
+          <t>280726145222415</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -16880,7 +16880,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C258" t="inlineStr"/>
@@ -16897,22 +16897,22 @@
       <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>280726145222634</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -16927,7 +16927,7 @@
       </c>
       <c r="M258" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N258" t="inlineStr">
@@ -16976,7 +16976,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>280726145221681</t>
+          <t>280726145222134</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>280726145222103</t>
+          <t>280726145222197</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -17072,7 +17072,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C261" t="inlineStr"/>
@@ -17089,22 +17089,22 @@
       <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>280726145221681</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -17119,7 +17119,7 @@
       </c>
       <c r="M261" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N261" t="inlineStr">
@@ -17168,7 +17168,7 @@
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>280726145222572</t>
+          <t>280726145222181</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
@@ -17200,7 +17200,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C263" t="inlineStr"/>
@@ -17217,22 +17217,22 @@
       <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>280726145222119</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -17247,7 +17247,7 @@
       </c>
       <c r="M263" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N263" t="inlineStr">
@@ -17296,7 +17296,7 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>280726145222415</t>
+          <t>280726145222572</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -17360,7 +17360,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>280726145222634</t>
+          <t>280726145222665</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -17424,7 +17424,7 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>280726145222134</t>
+          <t>280726145222447</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -17456,7 +17456,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C267" t="inlineStr"/>
@@ -17473,22 +17473,22 @@
       <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>280726145222650</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -17503,7 +17503,7 @@
       </c>
       <c r="M267" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N267" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145221697</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -17616,7 +17616,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>280726145222681</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -17680,7 +17680,7 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>280726145222197</t>
+          <t>280726145222650</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -17744,7 +17744,7 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>280726145222181</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>280726145221994</t>
+          <t>280726145222587</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -17872,7 +17872,7 @@
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>280726145222540</t>
+          <t>280726145222525</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -17936,7 +17936,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>280726145222165</t>
+          <t>280726145222322</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -17968,7 +17968,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C275" t="inlineStr"/>
@@ -17985,22 +17985,22 @@
       <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>280726145222009</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -18015,7 +18015,7 @@
       </c>
       <c r="M275" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N275" t="inlineStr">
@@ -18032,7 +18032,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C276" t="inlineStr"/>
@@ -18049,22 +18049,22 @@
       <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>280726145222494</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -18079,7 +18079,7 @@
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N276" t="inlineStr">
@@ -18096,7 +18096,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C277" t="inlineStr"/>
@@ -18113,22 +18113,22 @@
       <c r="F277" t="inlineStr"/>
       <c r="G277" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>280726145222494</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -18143,7 +18143,7 @@
       </c>
       <c r="M277" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N277" t="inlineStr">
@@ -18192,7 +18192,7 @@
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>280726145221697</t>
+          <t>280726145222337</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
@@ -18251,12 +18251,12 @@
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>280726145222290</t>
+          <t>280726145222228</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
@@ -18271,7 +18271,7 @@
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N279" t="inlineStr">
@@ -18384,7 +18384,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>280726145222337</t>
+          <t>280726145222697</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -18448,7 +18448,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>280726145222665</t>
+          <t>280726145222212</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -18512,7 +18512,7 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>280726145222619</t>
+          <t>280726145222165</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -18576,7 +18576,7 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222619</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -18640,7 +18640,7 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>280726145222587</t>
+          <t>280726145222540</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -18704,7 +18704,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>280726145222525</t>
+          <t>280726145222244</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -18768,7 +18768,7 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>280726145222322</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
@@ -18832,7 +18832,7 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>280726145222244</t>
+          <t>280726145222353</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -18896,7 +18896,7 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>280726145222212</t>
+          <t>280726145222150</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -18960,7 +18960,7 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>280726145222431</t>
+          <t>280726145222259</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -19019,12 +19019,12 @@
       </c>
       <c r="I291" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J291" t="inlineStr">
         <is>
-          <t>280726145222384</t>
+          <t>280726145222400</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
@@ -19039,7 +19039,7 @@
       </c>
       <c r="M291" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N291" t="inlineStr">
@@ -19056,7 +19056,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C292" t="inlineStr"/>
@@ -19073,22 +19073,22 @@
       <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J292" t="inlineStr">
         <is>
-          <t>280726145222400</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
@@ -19103,7 +19103,7 @@
       </c>
       <c r="M292" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N292" t="inlineStr">
@@ -19120,7 +19120,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C293" t="inlineStr"/>
@@ -19137,22 +19137,22 @@
       <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J293" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>280726145222306</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
@@ -19167,7 +19167,7 @@
       </c>
       <c r="M293" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N293" t="inlineStr">
@@ -19216,7 +19216,7 @@
       </c>
       <c r="J294" t="inlineStr">
         <is>
-          <t>280726145222259</t>
+          <t>280726145222431</t>
         </is>
       </c>
       <c r="K294" t="inlineStr">
@@ -19339,12 +19339,12 @@
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>33</t>
         </is>
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>280726145222306</t>
+          <t>280726145222384</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
@@ -19359,7 +19359,7 @@
       </c>
       <c r="M296" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>33</t>
         </is>
       </c>
       <c r="N296" t="inlineStr">
@@ -19440,7 +19440,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C298" t="inlineStr"/>
@@ -19457,27 +19457,27 @@
       <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr">
         <is>
-          <t>09/12/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>77</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>180626072347907</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L298" t="inlineStr">
@@ -19487,7 +19487,7 @@
       </c>
       <c r="M298" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>77</t>
         </is>
       </c>
       <c r="N298" t="inlineStr">
@@ -19504,7 +19504,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C299" t="inlineStr"/>
@@ -19521,27 +19521,27 @@
       <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>09/12/2031</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1944</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>110226132440294</t>
+          <t>180626072347907</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L299" t="inlineStr">
@@ -19551,7 +19551,7 @@
       </c>
       <c r="M299" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>50</t>
         </is>
       </c>
       <c r="N299" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 13/08/2026 08:57:56
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -747,12 +747,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -875,12 +875,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1195,12 +1195,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -1217,22 +1217,22 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1259,12 +1259,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -1281,22 +1281,22 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1675,12 +1675,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2507,12 +2507,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-002</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>120826061048781</t>
+          <t>120826061048765</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>120826061048765</t>
+          <t>120826061048718</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3019,12 +3019,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>120826061048718</t>
+          <t>120826061048781</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3243,12 +3243,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3280,7 +3280,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132440497</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3307,12 +3307,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-027-001-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3408,12 +3408,12 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132439966</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -3457,22 +3457,22 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3499,12 +3499,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-001-002</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -3536,12 +3536,12 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>110226132439966</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -3595,12 +3595,12 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3627,12 +3627,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132440497</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3777,22 +3777,22 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4097,22 +4097,22 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4203,12 +4203,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4353,22 +4353,22 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4417,22 +4417,22 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4481,22 +4481,22 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4737,22 +4737,22 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4843,12 +4843,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
@@ -4865,22 +4865,22 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132439700</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4939,12 +4939,12 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5099,12 +5099,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132439700</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5387,12 +5387,12 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6401,22 +6401,22 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6721,12 +6721,12 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7051,12 +7051,12 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7297,12 +7297,12 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7425,12 +7425,12 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7489,22 +7489,22 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7617,12 +7617,12 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7851,12 +7851,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8043,12 +8043,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8139,12 +8139,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8171,12 +8171,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8235,12 +8235,12 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C123" t="inlineStr"/>
@@ -8267,12 +8267,12 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8363,12 +8363,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9323,12 +9323,12 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C140" t="inlineStr"/>
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9409,22 +9409,22 @@
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9579,12 +9579,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C144" t="inlineStr"/>
@@ -9601,22 +9601,22 @@
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -10059,12 +10059,12 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10251,12 +10251,12 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>050826061104264</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050826061104264</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>050526131349498</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
@@ -11073,22 +11073,22 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
@@ -11120,7 +11120,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C168" t="inlineStr"/>
@@ -11137,22 +11137,22 @@
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050526131349498</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11248,7 +11248,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
@@ -11265,22 +11265,22 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11344,7 +11344,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11376,7 +11376,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C172" t="inlineStr"/>
@@ -11393,22 +11393,22 @@
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11521,12 +11521,12 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11777,22 +11777,22 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1993</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12033,22 +12033,22 @@
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
@@ -12097,22 +12097,22 @@
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12171,12 +12171,12 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12235,12 +12235,12 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12336,7 +12336,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
@@ -12353,22 +12353,22 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12491,12 +12491,12 @@
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12555,12 +12555,12 @@
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12747,12 +12747,12 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12801,22 +12801,22 @@
       <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1956</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -12875,12 +12875,12 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -12929,22 +12929,22 @@
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1956</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -12959,7 +12959,7 @@
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N196" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>300726064011668</t>
+          <t>300726064011918</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>300726064012981</t>
+          <t>300726064012543</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>300726064012543</t>
+          <t>300726064012575</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13360,7 +13360,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -13377,12 +13377,12 @@
       <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>300726064012668</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>300726064011997</t>
+          <t>300726064012684</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>300726064011887</t>
+          <t>300726064011997</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>300726064012825</t>
+          <t>300726064012715</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>300726064012637</t>
+          <t>300726064012934</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>300726064012575</t>
+          <t>300726064011981</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>300726064012903</t>
+          <t>300726064012622</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>300726064012731</t>
+          <t>300726064012012</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>300726064012512</t>
+          <t>300726064012637</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>300726064011856</t>
+          <t>300726064012512</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14064,7 +14064,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C214" t="inlineStr"/>
@@ -14081,22 +14081,22 @@
       <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>300726064011950</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14111,7 +14111,7 @@
       </c>
       <c r="M214" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>300726064011918</t>
+          <t>300726064012590</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>300726064012028</t>
+          <t>300726064012700</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>300726064013043</t>
+          <t>300726064011950</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>300726064012793</t>
+          <t>300726064012903</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -14416,7 +14416,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>300726064011965</t>
+          <t>300726064012106</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>300726064012918</t>
+          <t>300726064013012</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>300726064011653</t>
+          <t>300726064012856</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -14608,7 +14608,7 @@
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>300726064012809</t>
+          <t>300726064012825</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -14640,7 +14640,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C223" t="inlineStr"/>
@@ -14657,12 +14657,12 @@
       <c r="F223" t="inlineStr"/>
       <c r="G223" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>300726064012653</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -14704,7 +14704,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C224" t="inlineStr"/>
@@ -14721,22 +14721,22 @@
       <c r="F224" t="inlineStr"/>
       <c r="G224" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>300726064012497</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -14751,7 +14751,7 @@
       </c>
       <c r="M224" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N224" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>300726064012528</t>
+          <t>300726064012981</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>300726064013028</t>
+          <t>300726064012090</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14928,7 +14928,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>300726064012887</t>
+          <t>300726064012872</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -14992,7 +14992,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>300726064012965</t>
+          <t>300726064012559</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>300726064011934</t>
+          <t>300726064012731</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>300726064012559</t>
+          <t>300726064012997</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>300726064012872</t>
+          <t>300726064011668</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -15248,7 +15248,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>300726064012090</t>
+          <t>300726064011934</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15312,7 +15312,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>300726064012622</t>
+          <t>300726064012887</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15376,7 +15376,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>300726064012934</t>
+          <t>300726064012653</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>300726064012856</t>
+          <t>300726064012809</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15504,7 +15504,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>300726064012715</t>
+          <t>300726064011887</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -15568,7 +15568,7 @@
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>300726064013012</t>
+          <t>300726064013043</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15632,7 +15632,7 @@
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>300726064012106</t>
+          <t>300726064012028</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -15664,7 +15664,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C239" t="inlineStr"/>
@@ -15681,22 +15681,22 @@
       <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>300726064012793</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -15711,7 +15711,7 @@
       </c>
       <c r="M239" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N239" t="inlineStr">
@@ -15760,7 +15760,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>300726064012997</t>
+          <t>300726064011965</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -15824,7 +15824,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>300726064012700</t>
+          <t>300726064012965</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -15888,7 +15888,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>300726064011872</t>
+          <t>300726064012606</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -15952,7 +15952,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>300726064012122</t>
+          <t>300726064012950</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -16016,7 +16016,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>300726064012840</t>
+          <t>300726064012918</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16080,7 +16080,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>300726064012590</t>
+          <t>300726064011653</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -16112,7 +16112,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C246" t="inlineStr"/>
@@ -16129,22 +16129,22 @@
       <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>300726064013028</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -16159,7 +16159,7 @@
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N246" t="inlineStr">
@@ -16208,7 +16208,7 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>300726064012950</t>
+          <t>300726064012497</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -16272,7 +16272,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>300726064012606</t>
+          <t>300726064011856</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>300726064012012</t>
+          <t>300726064012840</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>300726064011981</t>
+          <t>300726064012122</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -16464,7 +16464,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>300726064012684</t>
+          <t>300726064011872</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -16528,7 +16528,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>300726064012668</t>
+          <t>300726064012528</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -16720,7 +16720,7 @@
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>280726145222181</t>
+          <t>280726145222509</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -16784,7 +16784,7 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>280726145222197</t>
+          <t>280726145222572</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>280726145222134</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -16912,7 +16912,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>280726145222634</t>
+          <t>280726145222650</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -16944,7 +16944,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C259" t="inlineStr"/>
@@ -16961,22 +16961,22 @@
       <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>280726145222478</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -16991,7 +16991,7 @@
       </c>
       <c r="M259" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N259" t="inlineStr">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>280726145222415</t>
+          <t>280726145222603</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -17104,7 +17104,7 @@
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>280726145221697</t>
+          <t>280726145222415</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -17168,7 +17168,7 @@
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>280726145222509</t>
+          <t>280726145222634</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
@@ -17232,7 +17232,7 @@
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>280726145222587</t>
+          <t>280726145222134</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -17296,7 +17296,7 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>280726145222572</t>
+          <t>280726145222197</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -17360,7 +17360,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>280726145222525</t>
+          <t>280726145222181</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -17392,7 +17392,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C266" t="inlineStr"/>
@@ -17409,22 +17409,22 @@
       <c r="F266" t="inlineStr"/>
       <c r="G266" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>280726145222322</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -17439,7 +17439,7 @@
       </c>
       <c r="M266" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N266" t="inlineStr">
@@ -17488,7 +17488,7 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>280726145222603</t>
+          <t>280726145221697</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>280726145222478</t>
+          <t>280726145222587</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -17616,7 +17616,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>280726145222650</t>
+          <t>280726145222525</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -17680,7 +17680,7 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222322</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>280726145222494</t>
+          <t>280726145222150</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -18064,7 +18064,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>280726145222150</t>
+          <t>280726145222353</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>280726145222353</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -18192,7 +18192,7 @@
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>280726145222697</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
@@ -18256,7 +18256,7 @@
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>280726145222697</t>
+          <t>280726145222228</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
@@ -18288,7 +18288,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C280" t="inlineStr"/>
@@ -18305,22 +18305,22 @@
       <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>280726145222228</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
@@ -18335,7 +18335,7 @@
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N280" t="inlineStr">
@@ -18352,7 +18352,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C281" t="inlineStr"/>
@@ -18369,22 +18369,22 @@
       <c r="F281" t="inlineStr"/>
       <c r="G281" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -18399,7 +18399,7 @@
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N281" t="inlineStr">
@@ -18416,7 +18416,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C282" t="inlineStr"/>
@@ -18433,22 +18433,22 @@
       <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>280726145222447</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -18463,7 +18463,7 @@
       </c>
       <c r="M282" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N282" t="inlineStr">
@@ -18480,7 +18480,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C283" t="inlineStr"/>
@@ -18497,22 +18497,22 @@
       <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>280726145222619</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -18527,7 +18527,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N283" t="inlineStr">
@@ -18576,7 +18576,7 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>280726145222447</t>
+          <t>280726145221681</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -18608,7 +18608,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C285" t="inlineStr"/>
@@ -18625,22 +18625,22 @@
       <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>280726145222103</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -18655,7 +18655,7 @@
       </c>
       <c r="M285" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N285" t="inlineStr">
@@ -18704,7 +18704,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>280726145221681</t>
+          <t>280726145222119</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -18768,7 +18768,7 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>280726145222244</t>
+          <t>280726145222681</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
@@ -18832,7 +18832,7 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>280726145222212</t>
+          <t>280726145221994</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -18896,7 +18896,7 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>280726145222103</t>
+          <t>280726145222009</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -18955,12 +18955,12 @@
       </c>
       <c r="I290" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>280726145222119</t>
+          <t>280726145222290</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -18975,7 +18975,7 @@
       </c>
       <c r="M290" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N290" t="inlineStr">
@@ -19024,7 +19024,7 @@
       </c>
       <c r="J291" t="inlineStr">
         <is>
-          <t>280726145222681</t>
+          <t>280726145222665</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
@@ -19088,7 +19088,7 @@
       </c>
       <c r="J292" t="inlineStr">
         <is>
-          <t>280726145221994</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
@@ -19152,7 +19152,7 @@
       </c>
       <c r="J293" t="inlineStr">
         <is>
-          <t>280726145222009</t>
+          <t>280726145222212</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
@@ -19211,12 +19211,12 @@
       </c>
       <c r="I294" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J294" t="inlineStr">
         <is>
-          <t>280726145222290</t>
+          <t>280726145222244</t>
         </is>
       </c>
       <c r="K294" t="inlineStr">
@@ -19231,7 +19231,7 @@
       </c>
       <c r="M294" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N294" t="inlineStr">
@@ -19280,7 +19280,7 @@
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222619</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
@@ -19344,7 +19344,7 @@
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>280726145222665</t>
+          <t>280726145222494</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
@@ -19376,7 +19376,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C297" t="inlineStr"/>
@@ -19393,22 +19393,22 @@
       <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J297" t="inlineStr">
         <is>
-          <t>280726145222306</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K297" t="inlineStr">
@@ -19423,7 +19423,7 @@
       </c>
       <c r="M297" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N297" t="inlineStr">
@@ -19504,7 +19504,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C299" t="inlineStr"/>
@@ -19521,22 +19521,22 @@
       <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>280726145222306</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -19551,7 +19551,7 @@
       </c>
       <c r="M299" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N299" t="inlineStr">
@@ -19664,7 +19664,7 @@
       </c>
       <c r="J301" t="inlineStr">
         <is>
-          <t>280726145222431</t>
+          <t>280726145222259</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
@@ -19728,7 +19728,7 @@
       </c>
       <c r="J302" t="inlineStr">
         <is>
-          <t>280726145222259</t>
+          <t>280726145222431</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 13/08/2026 10:00:58
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -2635,12 +2635,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>120826061048797</t>
+          <t>120826061048812</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>120826061048812</t>
+          <t>120826061048797</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-006-002</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>120826061048718</t>
+          <t>120826061048765</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-006-002</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>120826061048765</t>
+          <t>120826061048718</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3073,22 +3073,22 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3137,22 +3137,22 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3201,22 +3201,22 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3307,12 +3307,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132439700</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3393,22 +3393,22 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132439700</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3563,12 +3563,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132440497</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3627,12 +3627,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132440497</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3691,12 +3691,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3755,12 +3755,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -3777,22 +3777,22 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3947,12 +3947,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CAL-027-001-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -3984,12 +3984,12 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132439966</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -4011,12 +4011,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-001-002</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
@@ -4048,12 +4048,12 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>110226132439966</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 13/08/2026 10:27:23
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -17424,7 +17424,7 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>280726145222650</t>
+          <t>280726145222478</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -17488,7 +17488,7 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>280726145222478</t>
+          <t>280726145222650</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 13/08/2026 12:46:49
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -11536,7 +11536,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050826061104264</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>050826061104264</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>280726145222478</t>
+          <t>280726145222650</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -17616,7 +17616,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>280726145222650</t>
+          <t>280726145222478</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 13/08/2026 14:02:15
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -656,7 +656,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -715,12 +715,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -843,12 +843,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -907,12 +907,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1003,12 +1003,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1089,22 +1089,22 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2187,12 +2187,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2379,12 +2379,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3019,12 +3019,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>120826061048750</t>
+          <t>120826061048734</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3083,12 +3083,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>120826061048781</t>
+          <t>120826061048750</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048734</t>
+          <t>120826061048781</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3201,22 +3201,22 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3243,12 +3243,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3280,7 +3280,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132440497</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3393,22 +3393,22 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3435,12 +3435,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CAL-027-001-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -3472,12 +3472,12 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132439966</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3585,22 +3585,22 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3777,22 +3777,22 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3851,12 +3851,12 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3947,12 +3947,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -3969,22 +3969,22 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132439700</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4033,22 +4033,22 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4139,12 +4139,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132439700</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4225,22 +4225,22 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4289,22 +4289,22 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4481,22 +4481,22 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4523,12 +4523,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132440497</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4587,12 +4587,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-001-002</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -4624,12 +4624,12 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132439966</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4737,22 +4737,22 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4865,22 +4865,22 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5057,22 +5057,22 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5291,12 +5291,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6721,22 +6721,22 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7041,12 +7041,12 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,22 +7233,22 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7297,12 +7297,12 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7361,12 +7361,12 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7425,12 +7425,12 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7489,22 +7489,22 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7553,12 +7553,12 @@
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7617,12 +7617,12 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7681,12 +7681,12 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7755,12 +7755,12 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7775,7 +7775,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -7809,12 +7809,12 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8235,12 +8235,12 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C123" t="inlineStr"/>
@@ -8272,7 +8272,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8491,12 +8491,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8833,22 +8833,22 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8961,22 +8961,22 @@
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -10928,7 +10928,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
@@ -10945,22 +10945,22 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -11009,12 +11009,12 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1993</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>050826061104264</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
@@ -11073,22 +11073,22 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11344,7 +11344,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11457,12 +11457,12 @@
       <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>050826061104264</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11792,7 +11792,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12033,22 +12033,22 @@
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
@@ -12097,22 +12097,22 @@
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12208,7 +12208,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12363,12 +12363,12 @@
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12673,22 +12673,22 @@
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -12737,22 +12737,22 @@
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1956</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12801,22 +12801,22 @@
       <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1956</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -12875,12 +12875,12 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -12939,12 +12939,12 @@
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -12959,7 +12959,7 @@
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N196" t="inlineStr">
@@ -13168,7 +13168,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
@@ -13185,12 +13185,12 @@
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>300726064011950</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>300726064011887</t>
+          <t>300726064012903</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>300726064012981</t>
+          <t>300726064011997</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>300726064011997</t>
+          <t>300726064011856</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>300726064012903</t>
+          <t>300726064012637</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>300726064011668</t>
+          <t>300726064012512</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>300726064011950</t>
+          <t>300726064011903</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>300726064011856</t>
+          <t>300726064012981</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>300726064011903</t>
+          <t>300726064011887</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>300726064012825</t>
+          <t>300726064012575</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>300726064012637</t>
+          <t>300726064012731</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>300726064012575</t>
+          <t>300726064012543</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13936,7 +13936,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C212" t="inlineStr"/>
@@ -13953,12 +13953,12 @@
       <c r="F212" t="inlineStr"/>
       <c r="G212" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1826</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>300726064012731</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>300726064012543</t>
+          <t>300726064012825</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>300726064012512</t>
+          <t>300726064011918</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>300726064011918</t>
+          <t>300726064011668</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>280726145222650</t>
+          <t>280726145222478</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -17616,7 +17616,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>280726145222478</t>
+          <t>280726145222650</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 14/08/2026 06:03:08
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>1971</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>1971</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>1971</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>1971</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1847</t>
+          <t>1846</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1811</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1880</t>
+          <t>1879</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>1998</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>1998</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>1998</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>1998</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>1998</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>1998</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>1998</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1891</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1810</t>
+          <t>1809</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1810</t>
+          <t>1809</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1811</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1877</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1956</t>
+          <t>1955</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1993</t>
+          <t>1992</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1956</t>
+          <t>1955</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -13446,7 +13446,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -13766,7 +13766,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -14086,7 +14086,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -14150,7 +14150,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -14214,7 +14214,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -14278,7 +14278,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -14406,7 +14406,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -14534,7 +14534,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -14598,7 +14598,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
@@ -14662,7 +14662,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -14726,7 +14726,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -14790,7 +14790,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -14854,7 +14854,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -14918,7 +14918,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -15046,7 +15046,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -15110,7 +15110,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -15174,7 +15174,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
@@ -15238,7 +15238,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -15302,7 +15302,7 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
@@ -15430,7 +15430,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -15622,7 +15622,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -15686,7 +15686,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -15750,7 +15750,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -15814,7 +15814,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -15878,7 +15878,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -15942,7 +15942,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -16006,7 +16006,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
@@ -16070,7 +16070,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -16134,7 +16134,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
@@ -16198,7 +16198,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
@@ -16262,7 +16262,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -16326,7 +16326,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -16390,7 +16390,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -16582,7 +16582,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -16646,7 +16646,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -16774,7 +16774,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -16902,7 +16902,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -16966,7 +16966,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>1826</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -17030,7 +17030,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -17094,7 +17094,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
@@ -17158,7 +17158,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -17222,7 +17222,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
@@ -17350,7 +17350,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -17414,7 +17414,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -17478,7 +17478,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -17542,7 +17542,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -17606,7 +17606,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -17670,7 +17670,7 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
@@ -17734,7 +17734,7 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
@@ -17798,7 +17798,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -17862,7 +17862,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -17926,7 +17926,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -17990,7 +17990,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
@@ -18054,7 +18054,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -18118,7 +18118,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -18182,7 +18182,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -18246,7 +18246,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -18310,7 +18310,7 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
@@ -18374,7 +18374,7 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -18502,7 +18502,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -18566,7 +18566,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
@@ -18630,7 +18630,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
@@ -18758,7 +18758,7 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
@@ -18822,7 +18822,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
@@ -18886,7 +18886,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -18950,7 +18950,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
@@ -19014,7 +19014,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -19078,7 +19078,7 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
@@ -19142,7 +19142,7 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -19270,7 +19270,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -19334,7 +19334,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -19398,7 +19398,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -19462,7 +19462,7 @@
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
@@ -19526,7 +19526,7 @@
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -19590,7 +19590,7 @@
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
@@ -19654,7 +19654,7 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
@@ -19718,7 +19718,7 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -19782,7 +19782,7 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1891</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -19846,7 +19846,7 @@
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1926</t>
         </is>
       </c>
       <c r="I304" t="inlineStr">
@@ -19910,7 +19910,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -19974,7 +19974,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -20038,7 +20038,7 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
@@ -20102,7 +20102,7 @@
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>1996</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 14/08/2026 10:02:20
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -715,12 +715,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -779,12 +779,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1971</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1971</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -971,12 +971,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1089,22 +1089,22 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1971</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1971</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1867,12 +1867,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1931,12 +1931,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2187,12 +2187,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2443,12 +2443,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2507,12 +2507,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>120826061048734</t>
+          <t>120826061048781</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-006-002</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>120826061048765</t>
+          <t>120826061048718</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-027-006-002</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>120826061048750</t>
+          <t>120826061048765</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3083,12 +3083,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>120826061048781</t>
+          <t>120826061048750</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048718</t>
+          <t>120826061048734</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3179,12 +3179,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -3201,22 +3201,22 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3307,12 +3307,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132440497</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3435,12 +3435,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CAL-027-001-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -3457,27 +3457,27 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132439966</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3595,12 +3595,12 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3883,12 +3883,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -3905,22 +3905,22 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132440497</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3947,12 +3947,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-001-002</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -3984,12 +3984,12 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132439966</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -4033,22 +4033,22 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4289,22 +4289,22 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4523,12 +4523,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4971,12 +4971,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5121,22 +5121,22 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5185,22 +5185,22 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5227,12 +5227,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,22 +6081,22 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6209,22 +6209,22 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6239,7 +6239,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6401,12 +6401,12 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6465,12 +6465,12 @@
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6529,12 +6529,12 @@
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6657,12 +6657,12 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6721,12 +6721,12 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6785,12 +6785,12 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,12 +6913,12 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7041,22 +7041,22 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7169,12 +7169,12 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,12 +7233,12 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7297,12 +7297,12 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7435,12 +7435,12 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7489,12 +7489,12 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7553,12 +7553,12 @@
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7617,12 +7617,12 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7915,12 +7915,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C118" t="inlineStr"/>
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8043,12 +8043,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8427,12 +8427,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C126" t="inlineStr"/>
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8641,22 +8641,22 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8769,22 +8769,22 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1871</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9195,12 +9195,12 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9579,12 +9579,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C144" t="inlineStr"/>
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9995,12 +9995,12 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10187,12 +10187,12 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -10768,7 +10768,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050826061104264</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10800,7 +10800,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C163" t="inlineStr"/>
@@ -10817,22 +10817,22 @@
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>050526131349498</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11184,7 +11184,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C169" t="inlineStr"/>
@@ -11201,22 +11201,22 @@
       <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11265,12 +11265,12 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1992</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050526131349498</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11329,12 +11329,12 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1992</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11344,7 +11344,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11403,12 +11403,12 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>050826061104264</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11664,7 +11664,7 @@
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11792,7 +11792,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226062905996</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11856,7 +11856,7 @@
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>200226062905996</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12016,7 +12016,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C182" t="inlineStr"/>
@@ -12033,22 +12033,22 @@
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
@@ -12097,22 +12097,22 @@
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12144,7 +12144,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
@@ -12161,22 +12161,22 @@
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12208,7 +12208,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12673,22 +12673,22 @@
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1955</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -12747,12 +12747,12 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12801,22 +12801,22 @@
       <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1955</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -12875,12 +12875,12 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -12939,12 +12939,12 @@
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>44</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -12959,7 +12959,7 @@
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>44</t>
         </is>
       </c>
       <c r="N196" t="inlineStr">
@@ -13003,12 +13003,12 @@
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13023,7 +13023,7 @@
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N197" t="inlineStr">
@@ -13136,7 +13136,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>300726064011950</t>
+          <t>300726064011918</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13168,7 +13168,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
@@ -13185,12 +13185,12 @@
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>300726064012575</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>300726064012981</t>
+          <t>300726064011950</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>300726064012903</t>
+          <t>300726064012668</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>300726064012825</t>
+          <t>300726064012684</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>300726064011887</t>
+          <t>300726064012903</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>300726064011856</t>
+          <t>300726064011981</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>300726064012512</t>
+          <t>300726064012012</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13616,7 +13616,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C207" t="inlineStr"/>
@@ -13633,22 +13633,22 @@
       <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>300726064012637</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13663,7 +13663,7 @@
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N207" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>300726064012731</t>
+          <t>300726064011887</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>300726064012575</t>
+          <t>300726064012590</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>300726064011997</t>
+          <t>300726064012700</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>300726064012543</t>
+          <t>300726064011668</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>300726064011903</t>
+          <t>300726064012825</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>300726064011668</t>
+          <t>300726064012106</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>300726064011918</t>
+          <t>300726064013012</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>300726064013043</t>
+          <t>300726064012856</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>300726064012028</t>
+          <t>300726064012090</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>300726064012793</t>
+          <t>300726064012872</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>300726064011965</t>
+          <t>300726064011856</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -14416,7 +14416,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>300726064012918</t>
+          <t>300726064012559</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>300726064011653</t>
+          <t>300726064011934</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>300726064012809</t>
+          <t>300726064012887</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>300726064012497</t>
+          <t>300726064012809</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>300726064012528</t>
+          <t>300726064013043</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>300726064012887</t>
+          <t>300726064012543</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>300726064013028</t>
+          <t>300726064012028</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14928,7 +14928,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>300726064012965</t>
+          <t>300726064012793</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -14992,7 +14992,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>300726064011934</t>
+          <t>300726064011903</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>300726064012559</t>
+          <t>300726064011965</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>300726064012872</t>
+          <t>300726064011997</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>300726064012090</t>
+          <t>300726064012918</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -15248,7 +15248,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>300726064012622</t>
+          <t>300726064012637</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15312,7 +15312,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>300726064012934</t>
+          <t>300726064012512</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15376,7 +15376,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>300726064012856</t>
+          <t>300726064011653</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>300726064012715</t>
+          <t>300726064012497</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15504,7 +15504,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>300726064013012</t>
+          <t>300726064012528</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -15568,7 +15568,7 @@
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>300726064012106</t>
+          <t>300726064013028</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15600,7 +15600,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C238" t="inlineStr"/>
@@ -15617,22 +15617,22 @@
       <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>300726064012965</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -15647,7 +15647,7 @@
       </c>
       <c r="M238" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N238" t="inlineStr">
@@ -15696,7 +15696,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>300726064012997</t>
+          <t>300726064012840</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -15760,7 +15760,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>300726064012700</t>
+          <t>300726064012122</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -15824,7 +15824,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>300726064011872</t>
+          <t>300726064012950</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -15888,7 +15888,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>300726064012122</t>
+          <t>300726064012606</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -15920,7 +15920,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C243" t="inlineStr"/>
@@ -15937,12 +15937,12 @@
       <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -15952,7 +15952,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>300726064012840</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -16016,7 +16016,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>300726064012590</t>
+          <t>300726064011872</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16048,7 +16048,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C245" t="inlineStr"/>
@@ -16065,22 +16065,22 @@
       <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>300726064012981</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -16095,7 +16095,7 @@
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N245" t="inlineStr">
@@ -16144,7 +16144,7 @@
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>300726064012950</t>
+          <t>300726064012622</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -16208,7 +16208,7 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>300726064012606</t>
+          <t>300726064012934</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -16272,7 +16272,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>300726064012012</t>
+          <t>300726064012715</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>300726064011981</t>
+          <t>300726064012731</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>300726064012684</t>
+          <t>300726064012997</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -16432,7 +16432,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C251" t="inlineStr"/>
@@ -16449,22 +16449,22 @@
       <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>300726064012668</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -16479,7 +16479,7 @@
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N251" t="inlineStr">
@@ -16656,7 +16656,7 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>280726145222181</t>
+          <t>280726145221994</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -16720,7 +16720,7 @@
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>280726145222197</t>
+          <t>280726145222681</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -16784,7 +16784,7 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>280726145222134</t>
+          <t>280726145222478</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>280726145222634</t>
+          <t>280726145222603</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -16880,7 +16880,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C258" t="inlineStr"/>
@@ -16897,22 +16897,22 @@
       <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>280726145222009</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -16927,7 +16927,7 @@
       </c>
       <c r="M258" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N258" t="inlineStr">
@@ -16976,7 +16976,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>280726145222415</t>
+          <t>280726145222509</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>280726145221697</t>
+          <t>280726145222119</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -17104,7 +17104,7 @@
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>280726145222509</t>
+          <t>280726145222103</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -17163,12 +17163,12 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>280726145222572</t>
+          <t>280726145222290</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
@@ -17183,7 +17183,7 @@
       </c>
       <c r="M262" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N262" t="inlineStr">
@@ -17232,7 +17232,7 @@
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>280726145222587</t>
+          <t>280726145221681</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -17296,7 +17296,7 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>280726145222525</t>
+          <t>280726145222415</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -17360,7 +17360,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>280726145222322</t>
+          <t>280726145222634</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -17424,7 +17424,7 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>280726145222603</t>
+          <t>280726145222134</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -17456,7 +17456,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C267" t="inlineStr"/>
@@ -17473,22 +17473,22 @@
       <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>280726145222478</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -17503,7 +17503,7 @@
       </c>
       <c r="M267" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N267" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>280726145222650</t>
+          <t>280726145222197</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -17616,7 +17616,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222181</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -17680,7 +17680,7 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>280726145222337</t>
+          <t>280726145222572</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -17744,7 +17744,7 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>280726145222556</t>
+          <t>280726145222447</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>280726145222165</t>
+          <t>280726145222665</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -17840,7 +17840,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C273" t="inlineStr"/>
@@ -17857,22 +17857,22 @@
       <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>280726145222540</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -17887,7 +17887,7 @@
       </c>
       <c r="M273" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N273" t="inlineStr">
@@ -17936,7 +17936,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>280726145222494</t>
+          <t>280726145221697</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>280726145222150</t>
+          <t>280726145222650</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -18064,7 +18064,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>280726145222353</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -18192,7 +18192,7 @@
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>280726145222697</t>
+          <t>280726145222587</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
@@ -18256,7 +18256,7 @@
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>280726145222228</t>
+          <t>280726145222525</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
@@ -18320,7 +18320,7 @@
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>280726145222619</t>
+          <t>280726145222322</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
@@ -18352,7 +18352,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C281" t="inlineStr"/>
@@ -18369,22 +18369,22 @@
       <c r="F281" t="inlineStr"/>
       <c r="G281" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280726145222494</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -18399,7 +18399,7 @@
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N281" t="inlineStr">
@@ -18480,7 +18480,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C283" t="inlineStr"/>
@@ -18497,22 +18497,22 @@
       <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>280726145222447</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -18527,7 +18527,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N283" t="inlineStr">
@@ -18544,7 +18544,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C284" t="inlineStr"/>
@@ -18561,22 +18561,22 @@
       <c r="F284" t="inlineStr"/>
       <c r="G284" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>280726145222228</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N284" t="inlineStr">
@@ -18640,7 +18640,7 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>280726145222244</t>
+          <t>280726145222697</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -18704,7 +18704,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>280726145222212</t>
+          <t>280726145222337</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -18768,7 +18768,7 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>280726145221681</t>
+          <t>280726145222619</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
@@ -18832,7 +18832,7 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>280726145222103</t>
+          <t>280726145222556</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -18896,7 +18896,7 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>280726145222119</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -18960,7 +18960,7 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>280726145222681</t>
+          <t>280726145222353</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -19024,7 +19024,7 @@
       </c>
       <c r="J291" t="inlineStr">
         <is>
-          <t>280726145221994</t>
+          <t>280726145222212</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
@@ -19088,7 +19088,7 @@
       </c>
       <c r="J292" t="inlineStr">
         <is>
-          <t>280726145222009</t>
+          <t>280726145222165</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
@@ -19147,12 +19147,12 @@
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J293" t="inlineStr">
         <is>
-          <t>280726145222290</t>
+          <t>280726145222540</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
@@ -19167,7 +19167,7 @@
       </c>
       <c r="M293" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N293" t="inlineStr">
@@ -19216,7 +19216,7 @@
       </c>
       <c r="J294" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222244</t>
         </is>
       </c>
       <c r="K294" t="inlineStr">
@@ -19280,7 +19280,7 @@
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>280726145222665</t>
+          <t>280726145222150</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
@@ -19312,7 +19312,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C296" t="inlineStr"/>
@@ -19329,22 +19329,22 @@
       <c r="F296" t="inlineStr"/>
       <c r="G296" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>280726145222306</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
@@ -19359,7 +19359,7 @@
       </c>
       <c r="M296" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N296" t="inlineStr">
@@ -19403,12 +19403,12 @@
       </c>
       <c r="I297" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J297" t="inlineStr">
         <is>
-          <t>280726145222384</t>
+          <t>280726145222400</t>
         </is>
       </c>
       <c r="K297" t="inlineStr">
@@ -19423,7 +19423,7 @@
       </c>
       <c r="M297" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N297" t="inlineStr">
@@ -19440,7 +19440,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C298" t="inlineStr"/>
@@ -19457,22 +19457,22 @@
       <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>280726145222259</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
@@ -19487,7 +19487,7 @@
       </c>
       <c r="M298" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N298" t="inlineStr">
@@ -19536,7 +19536,7 @@
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>280726145222400</t>
+          <t>280726145222306</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -19632,7 +19632,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C301" t="inlineStr"/>
@@ -19649,22 +19649,22 @@
       <c r="F301" t="inlineStr"/>
       <c r="G301" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1891</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J301" t="inlineStr">
         <is>
-          <t>280726145222259</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
@@ -19679,7 +19679,7 @@
       </c>
       <c r="M301" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N301" t="inlineStr">
@@ -19696,7 +19696,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C302" t="inlineStr"/>
@@ -19713,22 +19713,22 @@
       <c r="F302" t="inlineStr"/>
       <c r="G302" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>33</t>
         </is>
       </c>
       <c r="J302" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>280726145222384</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
@@ -19743,7 +19743,7 @@
       </c>
       <c r="M302" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>33</t>
         </is>
       </c>
       <c r="N302" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 14/08/2026 12:46:22
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -523,7 +523,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 14/08/2026 13:49:19
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1971</t>
+          <t>1823</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -683,12 +683,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -705,22 +705,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1971</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1971</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1971</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -971,12 +971,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2955,12 +2955,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>120826061048734</t>
+          <t>120826061048718</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>120826061048718</t>
+          <t>120826061048750</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048750</t>
+          <t>120826061048734</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3457,22 +3457,22 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3585,22 +3585,22 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132440497</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3947,12 +3947,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-001-002</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -3969,27 +3969,27 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132439966</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4097,22 +4097,22 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4139,12 +4139,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440497</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4203,12 +4203,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CAL-027-001-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -4240,12 +4240,12 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132439966</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -4299,12 +4299,12 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4417,22 +4417,22 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4481,22 +4481,22 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4523,12 +4523,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4609,22 +4609,22 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4651,12 +4651,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
@@ -4673,22 +4673,22 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4715,12 +4715,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C68" t="inlineStr"/>
@@ -4737,22 +4737,22 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4971,12 +4971,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5035,12 +5035,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5227,12 +5227,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5313,22 +5313,22 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -5377,22 +5377,22 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,22 +6081,22 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6209,12 +6209,12 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6273,12 +6273,12 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6465,12 +6465,12 @@
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6593,12 +6593,12 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6721,12 +6721,12 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,12 +6913,12 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7041,22 +7041,22 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7307,12 +7307,12 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7425,12 +7425,12 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7489,12 +7489,12 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7563,12 +7563,12 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7745,12 +7745,12 @@
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7915,12 +7915,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C118" t="inlineStr"/>
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8203,12 +8203,12 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8395,12 +8395,12 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8641,22 +8641,22 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8961,22 +8961,22 @@
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1871</t>
+          <t>1928</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -9003,12 +9003,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9195,12 +9195,12 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -10059,12 +10059,12 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10187,12 +10187,12 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -11376,7 +11376,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C172" t="inlineStr"/>
@@ -11393,22 +11393,22 @@
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12208,7 +12208,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12737,22 +12737,22 @@
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1955</t>
+          <t>1825</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12801,22 +12801,22 @@
       <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1955</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -12875,12 +12875,12 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 15/08/2026 06:02:57
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1971</t>
+          <t>1970</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1971</t>
+          <t>1970</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1971</t>
+          <t>1970</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1971</t>
+          <t>1970</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1905</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1846</t>
+          <t>1845</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1811</t>
+          <t>1810</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1879</t>
+          <t>1878</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>1949</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>1949</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1809</t>
+          <t>1808</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1809</t>
+          <t>1808</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1811</t>
+          <t>1810</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1905</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1871</t>
+          <t>1870</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1928</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1877</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1955</t>
+          <t>1954</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1923</t>
+          <t>1922</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1923</t>
+          <t>1922</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1992</t>
+          <t>1991</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1891</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1955</t>
+          <t>1954</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -13446,7 +13446,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -13766,7 +13766,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -14086,7 +14086,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -14150,7 +14150,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -14214,7 +14214,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -14278,7 +14278,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -14406,7 +14406,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -14534,7 +14534,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -14598,7 +14598,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
@@ -14662,7 +14662,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -14726,7 +14726,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -14790,7 +14790,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -14854,7 +14854,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -14918,7 +14918,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -15046,7 +15046,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -15110,7 +15110,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -15174,7 +15174,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
@@ -15238,7 +15238,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -15302,7 +15302,7 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
@@ -15430,7 +15430,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -15622,7 +15622,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -15686,7 +15686,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -15750,7 +15750,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -15814,7 +15814,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -15878,7 +15878,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -15942,7 +15942,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -16006,7 +16006,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
@@ -16070,7 +16070,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -16134,7 +16134,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
@@ -16198,7 +16198,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
@@ -16262,7 +16262,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -16326,7 +16326,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -16390,7 +16390,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -16582,7 +16582,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -16646,7 +16646,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -16774,7 +16774,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -16902,7 +16902,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -16966,7 +16966,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -17030,7 +17030,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -17094,7 +17094,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
@@ -17158,7 +17158,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -17222,7 +17222,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
@@ -17350,7 +17350,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -17414,7 +17414,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -17478,7 +17478,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -17542,7 +17542,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -17606,7 +17606,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -17670,7 +17670,7 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
@@ -17734,7 +17734,7 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
@@ -17798,7 +17798,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -17862,7 +17862,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>1825</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -17926,7 +17926,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -17990,7 +17990,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
@@ -18054,7 +18054,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -18118,7 +18118,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -18182,7 +18182,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -18246,7 +18246,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -18310,7 +18310,7 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
@@ -18374,7 +18374,7 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -18502,7 +18502,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>1823</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -18566,7 +18566,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
@@ -18630,7 +18630,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
@@ -18758,7 +18758,7 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
@@ -18822,7 +18822,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
@@ -18886,7 +18886,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -18950,7 +18950,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
@@ -19014,7 +19014,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -19078,7 +19078,7 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
@@ -19142,7 +19142,7 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -19270,7 +19270,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -19334,7 +19334,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -19398,7 +19398,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -19462,7 +19462,7 @@
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
@@ -19526,7 +19526,7 @@
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -19590,7 +19590,7 @@
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
@@ -19654,7 +19654,7 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
@@ -19718,7 +19718,7 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -19782,7 +19782,7 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>1926</t>
+          <t>1925</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -19846,7 +19846,7 @@
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I304" t="inlineStr">
@@ -19910,7 +19910,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -19974,7 +19974,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -20038,7 +20038,7 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>1996</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 15/08/2026 07:30:40
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -18064,7 +18064,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 15/08/2026 07:43:10
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -18064,7 +18064,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 15/08/2026 08:33:24
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -18064,7 +18064,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 15/08/2026 08:45:55
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -18064,7 +18064,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 15/08/2026 11:41:25
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1970</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -683,12 +683,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -705,22 +705,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1970</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1970</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1970</t>
+          <t>1822</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -971,12 +971,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2955,12 +2955,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>120826061048718</t>
+          <t>120826061048734</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>120826061048750</t>
+          <t>120826061048718</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048734</t>
+          <t>120826061048750</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3457,22 +3457,22 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3585,22 +3585,22 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132440497</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3947,12 +3947,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CAL-027-001-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -3969,27 +3969,27 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132439966</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4097,22 +4097,22 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4139,12 +4139,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132440497</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4203,12 +4203,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-001-002</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -4240,12 +4240,12 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>110226132439966</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -4299,12 +4299,12 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4417,22 +4417,22 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4481,22 +4481,22 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4523,12 +4523,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4609,22 +4609,22 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4651,12 +4651,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
@@ -4673,22 +4673,22 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4715,12 +4715,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C68" t="inlineStr"/>
@@ -4737,22 +4737,22 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4971,12 +4971,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5035,12 +5035,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5227,12 +5227,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5313,22 +5313,22 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -5377,22 +5377,22 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,22 +6081,22 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6209,12 +6209,12 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6273,12 +6273,12 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6465,12 +6465,12 @@
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6593,12 +6593,12 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6721,12 +6721,12 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,12 +6913,12 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7041,22 +7041,22 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7307,12 +7307,12 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7425,12 +7425,12 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7489,12 +7489,12 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7563,12 +7563,12 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7745,12 +7745,12 @@
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7915,12 +7915,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C118" t="inlineStr"/>
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8203,12 +8203,12 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8395,12 +8395,12 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8641,22 +8641,22 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8961,22 +8961,22 @@
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1870</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -9003,12 +9003,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9195,12 +9195,12 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -10059,12 +10059,12 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10187,12 +10187,12 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -11376,7 +11376,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C172" t="inlineStr"/>
@@ -11393,22 +11393,22 @@
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12208,7 +12208,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12737,22 +12737,22 @@
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1954</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12801,22 +12801,22 @@
       <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1954</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -12875,12 +12875,12 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 18/08/2026 06:02:10
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1970</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1970</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1970</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1970</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1905</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1845</t>
+          <t>1842</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1810</t>
+          <t>1807</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1941</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1941</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1941</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1941</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1941</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1941</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1941</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1941</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1941</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1949</t>
+          <t>1946</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1949</t>
+          <t>1946</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1808</t>
+          <t>1805</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1808</t>
+          <t>1805</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1810</t>
+          <t>1807</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1905</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1954</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1922</t>
+          <t>1919</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1922</t>
+          <t>1919</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1991</t>
+          <t>1988</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1898</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1954</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -13446,7 +13446,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -13766,7 +13766,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -14086,7 +14086,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -14150,7 +14150,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -14214,7 +14214,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -14278,7 +14278,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -14406,7 +14406,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -14534,7 +14534,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -14598,7 +14598,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
@@ -14662,7 +14662,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -14726,7 +14726,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -14790,7 +14790,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -14854,7 +14854,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -14918,7 +14918,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -15046,7 +15046,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -15110,7 +15110,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -15174,7 +15174,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
@@ -15238,7 +15238,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -15302,7 +15302,7 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
@@ -15430,7 +15430,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -15622,7 +15622,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -15686,7 +15686,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -15750,7 +15750,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -15814,7 +15814,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -15878,7 +15878,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -15942,7 +15942,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -16006,7 +16006,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
@@ -16070,7 +16070,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -16134,7 +16134,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
@@ -16198,7 +16198,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
@@ -16262,7 +16262,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -16326,7 +16326,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -16390,7 +16390,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -16582,7 +16582,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -16646,7 +16646,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -16774,7 +16774,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -16902,7 +16902,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -16966,7 +16966,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -17030,7 +17030,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -17094,7 +17094,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
@@ -17158,7 +17158,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -17222,7 +17222,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
@@ -17350,7 +17350,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -17414,7 +17414,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -17478,7 +17478,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -17542,7 +17542,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -17606,7 +17606,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -17670,7 +17670,7 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
@@ -17734,7 +17734,7 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
@@ -17798,7 +17798,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -17862,7 +17862,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -17926,7 +17926,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -17990,7 +17990,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
@@ -18054,7 +18054,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -18118,7 +18118,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -18182,7 +18182,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -18246,7 +18246,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -18310,7 +18310,7 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
@@ -18374,7 +18374,7 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -18502,7 +18502,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>1822</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -18566,7 +18566,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
@@ -18630,7 +18630,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
@@ -18758,7 +18758,7 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
@@ -18822,7 +18822,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
@@ -18886,7 +18886,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -18950,7 +18950,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
@@ -19014,7 +19014,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -19078,7 +19078,7 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
@@ -19142,7 +19142,7 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -19270,7 +19270,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -19334,7 +19334,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -19398,7 +19398,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -19462,7 +19462,7 @@
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
@@ -19526,7 +19526,7 @@
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -19590,7 +19590,7 @@
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
@@ -19654,7 +19654,7 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
@@ -19718,7 +19718,7 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -19782,7 +19782,7 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>1925</t>
+          <t>1922</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -19846,7 +19846,7 @@
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I304" t="inlineStr">
@@ -19910,7 +19910,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1939</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -19974,7 +19974,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -20038,7 +20038,7 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>1992</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 18/08/2026 06:52:23
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -683,12 +683,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -705,22 +705,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -971,12 +971,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2955,12 +2955,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>120826061048734</t>
+          <t>120826061048718</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>120826061048718</t>
+          <t>120826061048750</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048750</t>
+          <t>120826061048734</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3457,22 +3457,22 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3585,22 +3585,22 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132440497</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3947,12 +3947,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-001-002</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -3969,27 +3969,27 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132439966</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4097,22 +4097,22 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4139,12 +4139,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440497</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4203,12 +4203,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CAL-027-001-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -4240,12 +4240,12 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132439966</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -4299,12 +4299,12 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4417,22 +4417,22 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4481,22 +4481,22 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4523,12 +4523,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4609,22 +4609,22 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4651,12 +4651,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
@@ -4673,22 +4673,22 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4715,12 +4715,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C68" t="inlineStr"/>
@@ -4737,22 +4737,22 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4971,12 +4971,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5035,12 +5035,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5227,12 +5227,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5313,22 +5313,22 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -5377,22 +5377,22 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,22 +6081,22 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6209,12 +6209,12 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6273,12 +6273,12 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6465,12 +6465,12 @@
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6593,12 +6593,12 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6721,12 +6721,12 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,12 +6913,12 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7041,22 +7041,22 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7307,12 +7307,12 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7425,12 +7425,12 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7489,12 +7489,12 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7563,12 +7563,12 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7745,12 +7745,12 @@
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7915,12 +7915,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C118" t="inlineStr"/>
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8203,12 +8203,12 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8395,12 +8395,12 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8641,22 +8641,22 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8961,22 +8961,22 @@
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -9003,12 +9003,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9195,12 +9195,12 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -10059,12 +10059,12 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10187,12 +10187,12 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -11376,7 +11376,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C172" t="inlineStr"/>
@@ -11393,22 +11393,22 @@
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12208,7 +12208,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12737,22 +12737,22 @@
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12801,22 +12801,22 @@
       <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -12875,12 +12875,12 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 18/08/2026 11:53:37
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -715,12 +715,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1003,12 +1003,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1099,12 +1099,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1547,12 +1547,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>120826061048812</t>
+          <t>120826061048797</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2827,12 +2827,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>120826061048797</t>
+          <t>120826061048812</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-006-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>120826061048765</t>
+          <t>120826061048781</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2955,12 +2955,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>120826061048750</t>
+          <t>120826061048734</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-006-002</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>120826061048718</t>
+          <t>120826061048765</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3083,12 +3083,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>120826061048781</t>
+          <t>120826061048718</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048734</t>
+          <t>120826061048750</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3435,12 +3435,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3585,22 +3585,22 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3691,12 +3691,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3755,12 +3755,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -3777,22 +3777,22 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3883,12 +3883,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4033,22 +4033,22 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4107,12 +4107,12 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4203,12 +4203,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -4225,22 +4225,22 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4363,12 +4363,12 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4427,12 +4427,12 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4459,12 +4459,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4523,12 +4523,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4907,12 +4907,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5121,22 +5121,22 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5697,27 +5697,27 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1807</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5761,27 +5761,27 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1807</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -5889,22 +5889,22 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,12 +6081,12 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6145,12 +6145,12 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6273,12 +6273,12 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6401,12 +6401,12 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,12 +6913,12 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6977,12 +6977,12 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7051,12 +7051,12 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7115,12 +7115,12 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7169,12 +7169,12 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,12 +7233,12 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7361,12 +7361,12 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7425,22 +7425,22 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7489,12 +7489,12 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7617,12 +7617,12 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7659,12 +7659,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7787,12 +7787,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7851,12 +7851,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8363,12 +8363,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8427,12 +8427,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C126" t="inlineStr"/>
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8577,22 +8577,22 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8769,22 +8769,22 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -10305,22 +10305,22 @@
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
-          <t>19/11/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1919</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>200226062756227</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -10369,22 +10369,22 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>19/11/2031</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1919</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226062756227</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>200226070819709</t>
+          <t>200226062756258</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>200226062756258</t>
+          <t>200226070819709</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -10689,22 +10689,22 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -10768,7 +10768,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050526131349498</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10928,7 +10928,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
@@ -10945,22 +10945,22 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>050526131349498</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
@@ -11585,22 +11585,22 @@
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11777,22 +11777,22 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11824,7 +11824,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
@@ -11841,22 +11841,22 @@
       <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
@@ -12097,22 +12097,22 @@
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12144,7 +12144,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
@@ -12161,22 +12161,22 @@
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12683,12 +12683,12 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -12747,12 +12747,12 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 18/08/2026 12:06:11
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -705,22 +705,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -784,7 +784,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1035,12 +1035,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1089,22 +1089,22 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1547,12 +1547,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2187,12 +2187,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2315,12 +2315,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2571,12 +2571,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>120826061048797</t>
+          <t>120826061048812</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2827,12 +2827,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>120826061048812</t>
+          <t>120826061048797</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>120826061048781</t>
+          <t>120826061048750</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048750</t>
+          <t>120826061048781</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3393,22 +3393,22 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3457,22 +3457,22 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3627,12 +3627,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3883,12 +3883,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -3905,22 +3905,22 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4011,12 +4011,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
@@ -4033,22 +4033,22 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4363,12 +4363,12 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4417,22 +4417,22 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4459,12 +4459,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -4481,22 +4481,22 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4523,12 +4523,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4609,22 +4609,22 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4651,12 +4651,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4875,12 +4875,12 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4907,12 +4907,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5057,22 +5057,22 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5099,12 +5099,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5185,22 +5185,22 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5259,12 +5259,12 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5279,7 +5279,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -5889,22 +5889,22 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,12 +6081,12 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6209,12 +6209,12 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6273,12 +6273,12 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6337,12 +6337,12 @@
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6721,12 +6721,12 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,12 +6913,12 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6977,12 +6977,12 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7051,12 +7051,12 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7169,12 +7169,12 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,12 +7233,12 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7297,12 +7297,12 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7361,12 +7361,12 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7425,22 +7425,22 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7489,12 +7489,12 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7563,12 +7563,12 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7617,12 +7617,12 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7659,12 +7659,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7851,12 +7851,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8171,12 +8171,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8363,12 +8363,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8491,12 +8491,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8577,22 +8577,22 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8769,22 +8769,22 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -10305,22 +10305,22 @@
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>19/11/2031</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1919</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226062756227</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -10369,22 +10369,22 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>19/11/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1919</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>200226062756227</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>200226062756258</t>
+          <t>200226070819709</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>200226070819709</t>
+          <t>200226062756258</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -10689,22 +10689,22 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -10768,7 +10768,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>050526131349498</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10928,7 +10928,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
@@ -10945,22 +10945,22 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050526131349498</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
@@ -11585,22 +11585,22 @@
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11777,22 +11777,22 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11824,7 +11824,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
@@ -11841,22 +11841,22 @@
       <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
@@ -12097,22 +12097,22 @@
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12144,7 +12144,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
@@ -12161,22 +12161,22 @@
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12683,12 +12683,12 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -12747,12 +12747,12 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -17936,7 +17936,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 18/08/2026 12:56:24
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -705,22 +705,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -784,7 +784,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1035,12 +1035,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1089,22 +1089,22 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1547,12 +1547,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2187,12 +2187,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2315,12 +2315,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2571,12 +2571,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>120826061048812</t>
+          <t>120826061048797</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2827,12 +2827,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>120826061048797</t>
+          <t>120826061048812</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>120826061048750</t>
+          <t>120826061048781</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048781</t>
+          <t>120826061048750</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3393,22 +3393,22 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3457,22 +3457,22 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3627,12 +3627,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3883,12 +3883,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -3905,22 +3905,22 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4011,12 +4011,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
@@ -4033,22 +4033,22 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4363,12 +4363,12 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4417,22 +4417,22 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4459,12 +4459,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -4481,22 +4481,22 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4523,12 +4523,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4609,22 +4609,22 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4651,12 +4651,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4875,12 +4875,12 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4907,12 +4907,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5057,22 +5057,22 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5099,12 +5099,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5185,22 +5185,22 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5259,12 +5259,12 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5279,7 +5279,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -5889,22 +5889,22 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,12 +6081,12 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6209,12 +6209,12 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6273,12 +6273,12 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6337,12 +6337,12 @@
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6721,12 +6721,12 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,12 +6913,12 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6977,12 +6977,12 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7051,12 +7051,12 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7169,12 +7169,12 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,12 +7233,12 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7297,12 +7297,12 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7361,12 +7361,12 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7425,22 +7425,22 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7489,12 +7489,12 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7563,12 +7563,12 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7617,12 +7617,12 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7659,12 +7659,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7851,12 +7851,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8171,12 +8171,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8363,12 +8363,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8491,12 +8491,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8577,22 +8577,22 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8769,22 +8769,22 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -10305,22 +10305,22 @@
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
-          <t>19/11/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1919</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>200226062756227</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -10369,22 +10369,22 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>19/11/2031</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1919</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226062756227</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>200226070819709</t>
+          <t>200226062756258</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>200226062756258</t>
+          <t>200226070819709</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -10689,22 +10689,22 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -10768,7 +10768,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050526131349498</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10928,7 +10928,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
@@ -10945,22 +10945,22 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>050526131349498</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
@@ -11585,22 +11585,22 @@
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11777,22 +11777,22 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11824,7 +11824,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
@@ -11841,22 +11841,22 @@
       <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
@@ -12097,22 +12097,22 @@
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12144,7 +12144,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
@@ -12161,22 +12161,22 @@
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12683,12 +12683,12 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -12747,12 +12747,12 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -17936,7 +17936,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 18/08/2026 13:44:37
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -715,12 +715,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1967</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1003,12 +1003,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1099,12 +1099,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1547,12 +1547,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>120826061048797</t>
+          <t>120826061048812</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2827,12 +2827,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>120826061048812</t>
+          <t>120826061048797</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-006-002</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>120826061048781</t>
+          <t>120826061048765</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2955,12 +2955,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>120826061048734</t>
+          <t>120826061048750</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-027-006-002</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>120826061048765</t>
+          <t>120826061048718</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3083,12 +3083,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>120826061048718</t>
+          <t>120826061048781</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048750</t>
+          <t>120826061048734</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3435,12 +3435,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3585,22 +3585,22 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3691,12 +3691,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3755,12 +3755,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -3777,22 +3777,22 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3883,12 +3883,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4033,22 +4033,22 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4107,12 +4107,12 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4203,12 +4203,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -4225,22 +4225,22 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519135</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4363,12 +4363,12 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4427,12 +4427,12 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4459,12 +4459,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4523,12 +4523,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130526104519135</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4907,12 +4907,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5121,22 +5121,22 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5697,27 +5697,27 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1807</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5761,27 +5761,27 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1807</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -5889,22 +5889,22 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,12 +6081,12 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6145,12 +6145,12 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6273,12 +6273,12 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6401,12 +6401,12 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,12 +6913,12 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6977,12 +6977,12 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7051,12 +7051,12 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7115,12 +7115,12 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7169,12 +7169,12 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,12 +7233,12 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7361,12 +7361,12 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7425,22 +7425,22 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7489,12 +7489,12 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7617,12 +7617,12 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7659,12 +7659,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7787,12 +7787,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7851,12 +7851,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8363,12 +8363,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8427,12 +8427,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C126" t="inlineStr"/>
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8577,22 +8577,22 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8769,22 +8769,22 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -10305,22 +10305,22 @@
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>19/11/2031</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1919</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226062756227</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -10369,22 +10369,22 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>19/11/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1919</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>200226062756227</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>200226062756258</t>
+          <t>200226070819709</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>200226070819709</t>
+          <t>200226062756258</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -10689,22 +10689,22 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -10768,7 +10768,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>050526131349498</t>
+          <t>050526131349561</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10928,7 +10928,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
@@ -10945,22 +10945,22 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>050526131349561</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050526131349498</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
@@ -11585,22 +11585,22 @@
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11777,22 +11777,22 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11824,7 +11824,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
@@ -11841,22 +11841,22 @@
       <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
@@ -12097,22 +12097,22 @@
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12144,7 +12144,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
@@ -12161,22 +12161,22 @@
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12683,12 +12683,12 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -12747,12 +12747,12 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 19/08/2026 06:02:49
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1841</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1807</t>
+          <t>1806</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1977</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1977</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1977</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1886</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1946</t>
+          <t>1945</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1946</t>
+          <t>1945</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1805</t>
+          <t>1804</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1805</t>
+          <t>1804</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1807</t>
+          <t>1806</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1919</t>
+          <t>1918</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1919</t>
+          <t>1918</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1988</t>
+          <t>1987</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -13446,7 +13446,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -13766,7 +13766,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -14086,7 +14086,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -14150,7 +14150,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -14214,7 +14214,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -14278,7 +14278,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -14406,7 +14406,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -14534,7 +14534,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -14598,7 +14598,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
@@ -14662,7 +14662,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -14726,7 +14726,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -14790,7 +14790,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -14854,7 +14854,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -14918,7 +14918,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -15046,7 +15046,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -15110,7 +15110,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -15174,7 +15174,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
@@ -15238,7 +15238,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -15302,7 +15302,7 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
@@ -15430,7 +15430,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -15622,7 +15622,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -15686,7 +15686,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -15750,7 +15750,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -15814,7 +15814,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -15878,7 +15878,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -15942,7 +15942,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -16006,7 +16006,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
@@ -16070,7 +16070,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -16134,7 +16134,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
@@ -16198,7 +16198,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
@@ -16262,7 +16262,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -16326,7 +16326,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -16390,7 +16390,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -16582,7 +16582,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -16646,7 +16646,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -16774,7 +16774,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -16902,7 +16902,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -16966,7 +16966,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -17030,7 +17030,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -17094,7 +17094,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
@@ -17158,7 +17158,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -17222,7 +17222,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
@@ -17350,7 +17350,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -17414,7 +17414,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -17478,7 +17478,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -17542,7 +17542,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -17606,7 +17606,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -17670,7 +17670,7 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
@@ -17734,7 +17734,7 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
@@ -17798,7 +17798,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -17862,7 +17862,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -17926,7 +17926,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -17990,7 +17990,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
@@ -18054,7 +18054,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -18118,7 +18118,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -18182,7 +18182,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -18246,7 +18246,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -18310,7 +18310,7 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
@@ -18374,7 +18374,7 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -18502,7 +18502,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -18566,7 +18566,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
@@ -18630,7 +18630,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
@@ -18758,7 +18758,7 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
@@ -18822,7 +18822,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
@@ -18886,7 +18886,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -18950,7 +18950,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
@@ -19014,7 +19014,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -19078,7 +19078,7 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
@@ -19142,7 +19142,7 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -19270,7 +19270,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -19334,7 +19334,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -19398,7 +19398,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -19462,7 +19462,7 @@
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
@@ -19526,7 +19526,7 @@
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1886</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -19590,7 +19590,7 @@
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
@@ -19654,7 +19654,7 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>1922</t>
+          <t>1921</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
@@ -19718,7 +19718,7 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -19782,7 +19782,7 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>1939</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -19846,7 +19846,7 @@
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I304" t="inlineStr">
@@ -19910,7 +19910,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>1992</t>
+          <t>1991</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 19/08/2026 10:04:20
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -1067,12 +1067,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1089,22 +1089,22 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>120826061048812</t>
+          <t>120826061048797</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2827,12 +2827,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>120826061048797</t>
+          <t>120826061048812</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3201,22 +3201,22 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3275,12 +3275,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3307,12 +3307,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3467,12 +3467,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3777,22 +3777,22 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3883,12 +3883,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3979,12 +3979,12 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4033,22 +4033,22 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4225,22 +4225,22 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4289,22 +4289,22 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4353,22 +4353,22 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4481,22 +4481,22 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4523,12 +4523,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4587,12 +4587,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4843,12 +4843,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
@@ -4865,22 +4865,22 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4929,22 +4929,22 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -4971,12 +4971,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5057,22 +5057,22 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5121,22 +5121,22 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5185,22 +5185,22 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5633,27 +5633,27 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1806</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -5697,27 +5697,27 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1806</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5825,12 +5825,12 @@
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5889,12 +5889,12 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6273,12 +6273,12 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6401,22 +6401,22 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6529,12 +6529,12 @@
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6593,12 +6593,12 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6657,12 +6657,12 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6721,12 +6721,12 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6785,12 +6785,12 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,12 +6913,12 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6977,22 +6977,22 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7041,12 +7041,12 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7105,12 +7105,12 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7297,12 +7297,12 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7371,12 +7371,12 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7489,22 +7489,22 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7659,12 +7659,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7723,12 +7723,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C115" t="inlineStr"/>
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8043,12 +8043,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8139,12 +8139,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8171,12 +8171,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8235,12 +8235,12 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C123" t="inlineStr"/>
@@ -8267,12 +8267,12 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8705,22 +8705,22 @@
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -8747,12 +8747,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C131" t="inlineStr"/>
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8897,22 +8897,22 @@
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1923</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8927,7 +8927,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N133" t="inlineStr">
@@ -10544,7 +10544,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
@@ -10561,22 +10561,22 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10591,7 +10591,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N159" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
@@ -10625,22 +10625,22 @@
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1987</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10655,7 +10655,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>300726064011950</t>
+          <t>300726064011668</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>300726064011668</t>
+          <t>300726064011950</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 19/08/2026 12:22:51
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -875,12 +875,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1089,22 +1089,22 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1163,12 +1163,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1547,12 +1547,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>120826061048797</t>
+          <t>120826061048812</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2827,12 +2827,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>120826061048812</t>
+          <t>120826061048797</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-006-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>120826061048765</t>
+          <t>120826061048734</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-006-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>120826061048718</t>
+          <t>120826061048765</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3019,12 +3019,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>120826061048781</t>
+          <t>120826061048718</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048734</t>
+          <t>120826061048781</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3275,12 +3275,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3435,12 +3435,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -3467,12 +3467,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3563,12 +3563,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3905,22 +3905,22 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3979,12 +3979,12 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4033,22 +4033,22 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4097,22 +4097,22 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4225,22 +4225,22 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4353,22 +4353,22 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4395,12 +4395,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4523,12 +4523,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4587,12 +4587,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -4609,22 +4609,22 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4843,12 +4843,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
@@ -4865,22 +4865,22 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4929,22 +4929,22 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5057,22 +5057,22 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5099,12 +5099,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -5121,22 +5121,22 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5185,22 +5185,22 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5633,27 +5633,27 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1806</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -5697,27 +5697,27 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1806</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5889,12 +5889,12 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6017,12 +6017,12 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6337,12 +6337,12 @@
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6657,12 +6657,12 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6721,12 +6721,12 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6785,12 +6785,12 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,22 +6913,22 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -6977,22 +6977,22 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7105,12 +7105,12 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,12 +7233,12 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7297,22 +7297,22 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7425,12 +7425,12 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7489,22 +7489,22 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7659,12 +7659,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7851,12 +7851,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8139,12 +8139,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8171,12 +8171,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8267,12 +8267,12 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8641,22 +8641,22 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1923</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8747,12 +8747,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C131" t="inlineStr"/>
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8897,22 +8897,22 @@
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8927,7 +8927,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9867,12 +9867,12 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9887,7 +9887,7 @@
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
@@ -9931,12 +9931,12 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -10448,7 +10448,7 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>200226070819709</t>
+          <t>200226062756258</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>200226062756258</t>
+          <t>200226070819709</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10544,7 +10544,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
@@ -10561,22 +10561,22 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050826061104264</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10591,7 +10591,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N159" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
@@ -10625,22 +10625,22 @@
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10655,7 +10655,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
@@ -10753,22 +10753,22 @@
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050826061104264</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11137,12 +11137,12 @@
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1987</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11248,7 +11248,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
@@ -11265,22 +11265,22 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11440,7 +11440,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C173" t="inlineStr"/>
@@ -11457,22 +11457,22 @@
       <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -11713,22 +11713,22 @@
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11777,22 +11777,22 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -12235,12 +12235,12 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12299,12 +12299,12 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12353,22 +12353,22 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12491,12 +12491,12 @@
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12619,12 +12619,12 @@
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12747,12 +12747,12 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>44</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>44</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12811,12 +12811,12 @@
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -12944,7 +12944,7 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>300726064011887</t>
+          <t>300726064011918</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -13008,7 +13008,7 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>300726064012981</t>
+          <t>300726064012575</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
@@ -13057,12 +13057,12 @@
       <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13072,7 +13072,7 @@
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>300726064011950</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -13136,7 +13136,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>300726064012903</t>
+          <t>300726064012668</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>300726064011668</t>
+          <t>300726064012684</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>300726064011950</t>
+          <t>300726064012903</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>300726064012825</t>
+          <t>300726064011981</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>300726064011856</t>
+          <t>300726064012012</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13424,7 +13424,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C204" t="inlineStr"/>
@@ -13441,22 +13441,22 @@
       <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1980</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>300726064012731</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13471,7 +13471,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N204" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>300726064012512</t>
+          <t>300726064011887</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>300726064012637</t>
+          <t>300726064012590</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>300726064011997</t>
+          <t>300726064012700</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>300726064012575</t>
+          <t>300726064011668</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>300726064011903</t>
+          <t>300726064012825</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>300726064012543</t>
+          <t>300726064012106</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>300726064011918</t>
+          <t>300726064013012</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>300726064013043</t>
+          <t>300726064012856</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>300726064012028</t>
+          <t>300726064012090</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>300726064012793</t>
+          <t>300726064011856</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>300726064011965</t>
+          <t>300726064012872</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>300726064012918</t>
+          <t>300726064012559</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>300726064011653</t>
+          <t>300726064011934</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>300726064012809</t>
+          <t>300726064012887</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>300726064012497</t>
+          <t>300726064012809</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>300726064012887</t>
+          <t>300726064012543</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -14608,7 +14608,7 @@
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>300726064012528</t>
+          <t>300726064013043</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>300726064013028</t>
+          <t>300726064012028</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>300726064012965</t>
+          <t>300726064011903</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>300726064011934</t>
+          <t>300726064012793</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>300726064012559</t>
+          <t>300726064011997</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14928,7 +14928,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>300726064012872</t>
+          <t>300726064011965</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -14992,7 +14992,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>300726064012090</t>
+          <t>300726064012918</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>300726064012622</t>
+          <t>300726064012637</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>300726064012934</t>
+          <t>300726064012512</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>300726064012856</t>
+          <t>300726064011653</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -15248,7 +15248,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>300726064012715</t>
+          <t>300726064012497</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15312,7 +15312,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>300726064013012</t>
+          <t>300726064012528</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15376,7 +15376,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>300726064012106</t>
+          <t>300726064013028</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -15408,7 +15408,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C235" t="inlineStr"/>
@@ -15425,22 +15425,22 @@
       <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>300726064012965</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15455,7 +15455,7 @@
       </c>
       <c r="M235" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N235" t="inlineStr">
@@ -15504,7 +15504,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>300726064012997</t>
+          <t>300726064012840</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -15568,7 +15568,7 @@
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>300726064012700</t>
+          <t>300726064012122</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15664,7 +15664,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C239" t="inlineStr"/>
@@ -15681,12 +15681,12 @@
       <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>1980</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -15696,7 +15696,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>300726064012122</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -15760,7 +15760,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>300726064012840</t>
+          <t>300726064012950</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -15824,7 +15824,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>300726064012590</t>
+          <t>300726064012981</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -15856,7 +15856,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C242" t="inlineStr"/>
@@ -15873,22 +15873,22 @@
       <c r="F242" t="inlineStr"/>
       <c r="G242" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>300726064012606</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -15903,7 +15903,7 @@
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N242" t="inlineStr">
@@ -15952,7 +15952,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>300726064012950</t>
+          <t>300726064012622</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -16016,7 +16016,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>300726064012012</t>
+          <t>300726064012934</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16080,7 +16080,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>300726064011981</t>
+          <t>300726064012731</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -16144,7 +16144,7 @@
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>300726064012606</t>
+          <t>300726064012997</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -16208,7 +16208,7 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>300726064012684</t>
+          <t>300726064012715</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -16240,7 +16240,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C248" t="inlineStr"/>
@@ -16257,22 +16257,22 @@
       <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>1980</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>300726064012668</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -16287,7 +16287,7 @@
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N248" t="inlineStr">
@@ -16464,7 +16464,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>280726145222181</t>
+          <t>280726145222681</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -16528,7 +16528,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>280726145222197</t>
+          <t>280726145221994</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>280726145222134</t>
+          <t>280726145222478</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -16656,7 +16656,7 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>280726145222634</t>
+          <t>280726145222603</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -16688,7 +16688,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C255" t="inlineStr"/>
@@ -16705,22 +16705,22 @@
       <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>280726145222009</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N255" t="inlineStr">
@@ -16784,7 +16784,7 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>280726145222415</t>
+          <t>280726145222509</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>280726145221697</t>
+          <t>280726145222119</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -16912,7 +16912,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>280726145222509</t>
+          <t>280726145222103</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -16976,7 +16976,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>280726145222572</t>
+          <t>280726145221681</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -17035,12 +17035,12 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>280726145222587</t>
+          <t>280726145222290</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -17055,7 +17055,7 @@
       </c>
       <c r="M260" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N260" t="inlineStr">
@@ -17104,7 +17104,7 @@
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>280726145222525</t>
+          <t>280726145222415</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -17168,7 +17168,7 @@
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>280726145222650</t>
+          <t>280726145222634</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
@@ -17232,7 +17232,7 @@
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>280726145222603</t>
+          <t>280726145222134</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -17264,7 +17264,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C264" t="inlineStr"/>
@@ -17281,22 +17281,22 @@
       <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>280726145222478</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -17311,7 +17311,7 @@
       </c>
       <c r="M264" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N264" t="inlineStr">
@@ -17360,7 +17360,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222197</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -17424,7 +17424,7 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>280726145222322</t>
+          <t>280726145222181</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -17488,7 +17488,7 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>280726145222337</t>
+          <t>280726145222572</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>280726145222556</t>
+          <t>280726145222447</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -17584,7 +17584,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C269" t="inlineStr"/>
@@ -17601,22 +17601,22 @@
       <c r="F269" t="inlineStr"/>
       <c r="G269" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>280726145222165</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -17631,7 +17631,7 @@
       </c>
       <c r="M269" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N269" t="inlineStr">
@@ -17680,7 +17680,7 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>280726145222540</t>
+          <t>280726145222665</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -17744,7 +17744,7 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>280726145222494</t>
+          <t>280726145221697</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>280726145222150</t>
+          <t>280726145222650</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -17872,7 +17872,7 @@
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>280726145222353</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -17936,7 +17936,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>280726145222619</t>
+          <t>280726145222587</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -18064,7 +18064,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>280726145222697</t>
+          <t>280726145222525</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>280726145222228</t>
+          <t>280726145222322</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -18160,7 +18160,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C278" t="inlineStr"/>
@@ -18177,22 +18177,22 @@
       <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280726145222494</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
@@ -18207,7 +18207,7 @@
       </c>
       <c r="M278" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N278" t="inlineStr">
@@ -18288,7 +18288,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C280" t="inlineStr"/>
@@ -18305,22 +18305,22 @@
       <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>280726145222244</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
@@ -18335,7 +18335,7 @@
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N280" t="inlineStr">
@@ -18384,7 +18384,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>280726145222212</t>
+          <t>280726145222228</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -18448,7 +18448,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>280726145222447</t>
+          <t>280726145222697</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -18480,7 +18480,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C283" t="inlineStr"/>
@@ -18497,22 +18497,22 @@
       <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>280726145222337</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -18527,7 +18527,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N283" t="inlineStr">
@@ -18576,7 +18576,7 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>280726145221681</t>
+          <t>280726145222619</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -18640,7 +18640,7 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>280726145222103</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -18704,7 +18704,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>280726145222119</t>
+          <t>280726145222353</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -18768,7 +18768,7 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>280726145222681</t>
+          <t>280726145222556</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
@@ -18832,7 +18832,7 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>280726145221994</t>
+          <t>280726145222150</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -18896,7 +18896,7 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>280726145222009</t>
+          <t>280726145222165</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -18960,7 +18960,7 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222540</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -19019,12 +19019,12 @@
       </c>
       <c r="I291" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J291" t="inlineStr">
         <is>
-          <t>280726145222290</t>
+          <t>280726145222212</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
@@ -19039,7 +19039,7 @@
       </c>
       <c r="M291" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N291" t="inlineStr">
@@ -19088,7 +19088,7 @@
       </c>
       <c r="J292" t="inlineStr">
         <is>
-          <t>280726145222665</t>
+          <t>280726145222244</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
@@ -19120,7 +19120,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C293" t="inlineStr"/>
@@ -19137,22 +19137,22 @@
       <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J293" t="inlineStr">
         <is>
-          <t>280726145222306</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
@@ -19167,7 +19167,7 @@
       </c>
       <c r="M293" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N293" t="inlineStr">
@@ -19211,12 +19211,12 @@
       </c>
       <c r="I294" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J294" t="inlineStr">
         <is>
-          <t>280726145222384</t>
+          <t>280726145222400</t>
         </is>
       </c>
       <c r="K294" t="inlineStr">
@@ -19231,7 +19231,7 @@
       </c>
       <c r="M294" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N294" t="inlineStr">
@@ -19248,7 +19248,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C295" t="inlineStr"/>
@@ -19265,22 +19265,22 @@
       <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>280726145222259</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
@@ -19295,7 +19295,7 @@
       </c>
       <c r="M295" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N295" t="inlineStr">
@@ -19344,7 +19344,7 @@
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>280726145222400</t>
+          <t>280726145222306</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
@@ -19440,7 +19440,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C298" t="inlineStr"/>
@@ -19457,22 +19457,22 @@
       <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1886</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>280726145222259</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
@@ -19487,7 +19487,7 @@
       </c>
       <c r="M298" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N298" t="inlineStr">
@@ -19504,7 +19504,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C299" t="inlineStr"/>
@@ -19521,22 +19521,22 @@
       <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>1886</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>33</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>280726145222384</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -19551,7 +19551,7 @@
       </c>
       <c r="M299" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>33</t>
         </is>
       </c>
       <c r="N299" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 19/08/2026 15:31:28
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -875,12 +875,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1089,22 +1089,22 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1163,12 +1163,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1547,12 +1547,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>120826061048812</t>
+          <t>120826061048797</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2827,12 +2827,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>120826061048797</t>
+          <t>120826061048812</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-006-002</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>120826061048734</t>
+          <t>120826061048765</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-006-002</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>120826061048765</t>
+          <t>120826061048718</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3019,12 +3019,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>120826061048718</t>
+          <t>120826061048781</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048781</t>
+          <t>120826061048734</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3275,12 +3275,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3435,12 +3435,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -3467,12 +3467,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3563,12 +3563,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132440372</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3905,22 +3905,22 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3979,12 +3979,12 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4033,22 +4033,22 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4097,22 +4097,22 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4225,22 +4225,22 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4353,22 +4353,22 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4395,12 +4395,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4523,12 +4523,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>110226132440372</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4587,12 +4587,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -4609,22 +4609,22 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4843,12 +4843,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
@@ -4865,22 +4865,22 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4929,22 +4929,22 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5057,22 +5057,22 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5099,12 +5099,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -5121,22 +5121,22 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5185,22 +5185,22 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5633,27 +5633,27 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1806</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -5697,27 +5697,27 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1806</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5889,12 +5889,12 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6017,12 +6017,12 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6337,12 +6337,12 @@
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6657,12 +6657,12 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6721,12 +6721,12 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6785,12 +6785,12 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6849,12 +6849,12 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,22 +6913,22 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -6977,22 +6977,22 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7105,12 +7105,12 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,12 +7233,12 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7297,22 +7297,22 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7425,12 +7425,12 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7489,22 +7489,22 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7659,12 +7659,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7851,12 +7851,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8139,12 +8139,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8171,12 +8171,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8267,12 +8267,12 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8641,22 +8641,22 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8747,12 +8747,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C131" t="inlineStr"/>
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8897,22 +8897,22 @@
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1923</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8927,7 +8927,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9867,12 +9867,12 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9887,7 +9887,7 @@
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
@@ -9931,12 +9931,12 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -10448,7 +10448,7 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>200226062756258</t>
+          <t>200226070819709</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>200226070819709</t>
+          <t>200226062756258</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10544,7 +10544,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
@@ -10561,22 +10561,22 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>050826061104264</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10591,7 +10591,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N159" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
@@ -10625,22 +10625,22 @@
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1987</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10655,7 +10655,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
@@ -10753,22 +10753,22 @@
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>050826061104295</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>050826061104295</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050826061104264</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11137,12 +11137,12 @@
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11248,7 +11248,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
@@ -11265,22 +11265,22 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11440,7 +11440,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C173" t="inlineStr"/>
@@ -11457,22 +11457,22 @@
       <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -11713,22 +11713,22 @@
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11777,22 +11777,22 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -12235,12 +12235,12 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12299,12 +12299,12 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12353,22 +12353,22 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12491,12 +12491,12 @@
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12619,12 +12619,12 @@
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12747,12 +12747,12 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12811,12 +12811,12 @@
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>44</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>44</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -12944,7 +12944,7 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>300726064011918</t>
+          <t>300726064011887</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -13008,7 +13008,7 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>300726064012575</t>
+          <t>300726064012981</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
@@ -13057,12 +13057,12 @@
       <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1980</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13072,7 +13072,7 @@
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>300726064011950</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -13136,7 +13136,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>300726064012668</t>
+          <t>300726064012903</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>300726064012684</t>
+          <t>300726064011668</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>300726064012903</t>
+          <t>300726064011950</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>300726064011981</t>
+          <t>300726064012825</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>300726064012012</t>
+          <t>300726064011856</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13424,7 +13424,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C204" t="inlineStr"/>
@@ -13441,22 +13441,22 @@
       <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>300726064012731</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13471,7 +13471,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N204" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>300726064011887</t>
+          <t>300726064012512</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>300726064012590</t>
+          <t>300726064012637</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>300726064012700</t>
+          <t>300726064011997</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>300726064011668</t>
+          <t>300726064012575</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>300726064012825</t>
+          <t>300726064011903</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>300726064012106</t>
+          <t>300726064012543</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>300726064013012</t>
+          <t>300726064011918</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>300726064012856</t>
+          <t>300726064013043</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>300726064012090</t>
+          <t>300726064012028</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>300726064011856</t>
+          <t>300726064012793</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>300726064012872</t>
+          <t>300726064011965</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>300726064012559</t>
+          <t>300726064012918</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>300726064011934</t>
+          <t>300726064011653</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>300726064012887</t>
+          <t>300726064012809</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>300726064012809</t>
+          <t>300726064012497</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>300726064012543</t>
+          <t>300726064012887</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -14608,7 +14608,7 @@
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>300726064013043</t>
+          <t>300726064012528</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>300726064012028</t>
+          <t>300726064013028</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>300726064011903</t>
+          <t>300726064012965</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>300726064012793</t>
+          <t>300726064011934</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>300726064011997</t>
+          <t>300726064012559</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14928,7 +14928,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>300726064011965</t>
+          <t>300726064012872</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -14992,7 +14992,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>300726064012918</t>
+          <t>300726064012090</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>300726064012637</t>
+          <t>300726064012622</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>300726064012512</t>
+          <t>300726064012934</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>300726064011653</t>
+          <t>300726064012856</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -15248,7 +15248,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>300726064012497</t>
+          <t>300726064012715</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15312,7 +15312,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>300726064012528</t>
+          <t>300726064013012</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15376,7 +15376,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>300726064013028</t>
+          <t>300726064012106</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -15408,7 +15408,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C235" t="inlineStr"/>
@@ -15425,22 +15425,22 @@
       <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>1980</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>300726064012965</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15455,7 +15455,7 @@
       </c>
       <c r="M235" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N235" t="inlineStr">
@@ -15504,7 +15504,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>300726064012840</t>
+          <t>300726064012997</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -15568,7 +15568,7 @@
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>300726064012122</t>
+          <t>300726064012700</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15664,7 +15664,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C239" t="inlineStr"/>
@@ -15681,12 +15681,12 @@
       <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -15696,7 +15696,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>300726064012122</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -15760,7 +15760,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>300726064012950</t>
+          <t>300726064012840</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -15824,7 +15824,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>300726064012981</t>
+          <t>300726064012590</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -15856,7 +15856,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C242" t="inlineStr"/>
@@ -15873,22 +15873,22 @@
       <c r="F242" t="inlineStr"/>
       <c r="G242" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>1980</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>300726064012606</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -15903,7 +15903,7 @@
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N242" t="inlineStr">
@@ -15952,7 +15952,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>300726064012622</t>
+          <t>300726064012950</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -16016,7 +16016,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>300726064012934</t>
+          <t>300726064012012</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16080,7 +16080,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>300726064012731</t>
+          <t>300726064011981</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -16144,7 +16144,7 @@
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>300726064012997</t>
+          <t>300726064012606</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -16208,7 +16208,7 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>300726064012715</t>
+          <t>300726064012684</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -16240,7 +16240,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C248" t="inlineStr"/>
@@ -16257,22 +16257,22 @@
       <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>300726064012668</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -16287,7 +16287,7 @@
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N248" t="inlineStr">
@@ -16464,7 +16464,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>280726145222681</t>
+          <t>280726145222181</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -16528,7 +16528,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>280726145221994</t>
+          <t>280726145222197</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>280726145222478</t>
+          <t>280726145222134</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -16656,7 +16656,7 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>280726145222603</t>
+          <t>280726145222634</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -16688,7 +16688,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C255" t="inlineStr"/>
@@ -16705,22 +16705,22 @@
       <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1820</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>280726145222009</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N255" t="inlineStr">
@@ -16784,7 +16784,7 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>280726145222509</t>
+          <t>280726145222415</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>280726145222119</t>
+          <t>280726145221697</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -16912,7 +16912,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>280726145222103</t>
+          <t>280726145222509</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -16976,7 +16976,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>280726145221681</t>
+          <t>280726145222572</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -17035,12 +17035,12 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>280726145222290</t>
+          <t>280726145222587</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -17055,7 +17055,7 @@
       </c>
       <c r="M260" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N260" t="inlineStr">
@@ -17104,7 +17104,7 @@
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>280726145222415</t>
+          <t>280726145222525</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -17168,7 +17168,7 @@
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>280726145222634</t>
+          <t>280726145222650</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
@@ -17232,7 +17232,7 @@
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>280726145222134</t>
+          <t>280726145222603</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -17264,7 +17264,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C264" t="inlineStr"/>
@@ -17281,22 +17281,22 @@
       <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>280726145222478</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -17311,7 +17311,7 @@
       </c>
       <c r="M264" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N264" t="inlineStr">
@@ -17360,7 +17360,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>280726145222197</t>
+          <t>280726145222462</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -17424,7 +17424,7 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>280726145222181</t>
+          <t>280726145222322</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -17488,7 +17488,7 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>280726145222572</t>
+          <t>280726145222337</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>280726145222447</t>
+          <t>280726145222556</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -17584,7 +17584,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C269" t="inlineStr"/>
@@ -17601,22 +17601,22 @@
       <c r="F269" t="inlineStr"/>
       <c r="G269" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>280726145222165</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -17631,7 +17631,7 @@
       </c>
       <c r="M269" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N269" t="inlineStr">
@@ -17680,7 +17680,7 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>280726145222665</t>
+          <t>280726145222540</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -17744,7 +17744,7 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>280726145221697</t>
+          <t>280726145222494</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>280726145222650</t>
+          <t>280726145222150</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -17872,7 +17872,7 @@
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>280726145222462</t>
+          <t>280726145222353</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -17936,7 +17936,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>280726145222587</t>
+          <t>280726145222619</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>280726145222025</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -18064,7 +18064,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>280726145222525</t>
+          <t>280726145222697</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>280726145222322</t>
+          <t>280726145222228</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -18160,7 +18160,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C278" t="inlineStr"/>
@@ -18177,22 +18177,22 @@
       <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>280726145222494</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
@@ -18207,7 +18207,7 @@
       </c>
       <c r="M278" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N278" t="inlineStr">
@@ -18288,7 +18288,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C280" t="inlineStr"/>
@@ -18305,22 +18305,22 @@
       <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280726145222244</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
@@ -18335,7 +18335,7 @@
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N280" t="inlineStr">
@@ -18384,7 +18384,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>280726145222228</t>
+          <t>280726145222212</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -18448,7 +18448,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>280726145222697</t>
+          <t>280726145222447</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -18480,7 +18480,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C283" t="inlineStr"/>
@@ -18497,22 +18497,22 @@
       <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>280726145222337</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -18527,7 +18527,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N283" t="inlineStr">
@@ -18576,7 +18576,7 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>280726145222619</t>
+          <t>280726145221681</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -18640,7 +18640,7 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>280726145222103</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -18704,7 +18704,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>280726145222353</t>
+          <t>280726145222119</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -18768,7 +18768,7 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>280726145222556</t>
+          <t>280726145222681</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
@@ -18832,7 +18832,7 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>280726145222150</t>
+          <t>280726145221994</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -18896,7 +18896,7 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>280726145222165</t>
+          <t>280726145222009</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -18960,7 +18960,7 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>280726145222540</t>
+          <t>280726145222025</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -19019,12 +19019,12 @@
       </c>
       <c r="I291" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J291" t="inlineStr">
         <is>
-          <t>280726145222212</t>
+          <t>280726145222290</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
@@ -19039,7 +19039,7 @@
       </c>
       <c r="M291" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N291" t="inlineStr">
@@ -19088,7 +19088,7 @@
       </c>
       <c r="J292" t="inlineStr">
         <is>
-          <t>280726145222244</t>
+          <t>280726145222665</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
@@ -19120,7 +19120,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C293" t="inlineStr"/>
@@ -19137,22 +19137,22 @@
       <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J293" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>280726145222306</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
@@ -19167,7 +19167,7 @@
       </c>
       <c r="M293" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N293" t="inlineStr">
@@ -19211,12 +19211,12 @@
       </c>
       <c r="I294" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>33</t>
         </is>
       </c>
       <c r="J294" t="inlineStr">
         <is>
-          <t>280726145222400</t>
+          <t>280726145222384</t>
         </is>
       </c>
       <c r="K294" t="inlineStr">
@@ -19231,7 +19231,7 @@
       </c>
       <c r="M294" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>33</t>
         </is>
       </c>
       <c r="N294" t="inlineStr">
@@ -19248,7 +19248,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C295" t="inlineStr"/>
@@ -19265,22 +19265,22 @@
       <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>280726145222259</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
@@ -19295,7 +19295,7 @@
       </c>
       <c r="M295" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N295" t="inlineStr">
@@ -19344,7 +19344,7 @@
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>280726145222306</t>
+          <t>280726145222400</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
@@ -19440,7 +19440,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C298" t="inlineStr"/>
@@ -19457,22 +19457,22 @@
       <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>1886</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>280726145222259</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
@@ -19487,7 +19487,7 @@
       </c>
       <c r="M298" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N298" t="inlineStr">
@@ -19504,7 +19504,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C299" t="inlineStr"/>
@@ -19521,22 +19521,22 @@
       <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1886</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>280726145222384</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -19551,7 +19551,7 @@
       </c>
       <c r="M299" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N299" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 20/08/2026 07:30:20
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1965</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -683,12 +683,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -705,22 +705,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1965</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -912,7 +912,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1965</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1965</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -1089,22 +1089,22 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1153,22 +1153,22 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>62</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1867,12 +1867,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1931,12 +1931,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2379,12 +2379,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>120826061048812</t>
+          <t>120826061048797</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>2399</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2827,12 +2827,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>120826061048797</t>
+          <t>120826061048812</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2399</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-006-002</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2891,12 +2891,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>120826061048781</t>
+          <t>120826061048765</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>120826061048750</t>
+          <t>120826061048718</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3019,12 +3019,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>120826061048718</t>
+          <t>120826061048781</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3083,12 +3083,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>120826061048734</t>
+          <t>120826061048750</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-006-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048765</t>
+          <t>120826061048734</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3211,12 +3211,12 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3243,12 +3243,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3280,7 +3280,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3393,22 +3393,22 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3457,22 +3457,22 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3563,12 +3563,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3905,22 +3905,22 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3969,22 +3969,22 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4075,12 +4075,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C58" t="inlineStr"/>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4289,22 +4289,22 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4353,22 +4353,22 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4395,12 +4395,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -4417,22 +4417,22 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4459,12 +4459,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4587,12 +4587,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4673,22 +4673,22 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5057,22 +5057,22 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5121,22 +5121,22 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5569,27 +5569,27 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1805</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -5599,7 +5599,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5633,27 +5633,27 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1805</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -5761,12 +5761,12 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5825,12 +5825,12 @@
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6027,12 +6027,12 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6081,22 +6081,22 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6145,12 +6145,12 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6209,12 +6209,12 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6337,12 +6337,12 @@
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6465,12 +6465,12 @@
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6529,12 +6529,12 @@
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6657,22 +6657,22 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6785,12 +6785,12 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7105,22 +7105,22 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7169,12 +7169,12 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7297,12 +7297,12 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7425,12 +7425,12 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7627,12 +7627,12 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7787,12 +7787,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
@@ -7819,12 +7819,12 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -7851,12 +7851,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8043,12 +8043,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8107,12 +8107,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8577,22 +8577,22 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1865</t>
+          <t>1922</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8683,12 +8683,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C130" t="inlineStr"/>
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8833,22 +8833,22 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1922</t>
+          <t>1865</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9003,12 +9003,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9803,12 +9803,12 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N147" t="inlineStr">
@@ -9867,12 +9867,12 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9887,7 +9887,7 @@
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
@@ -10177,22 +10177,22 @@
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
-          <t>19/11/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1917</t>
+          <t>1949</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>200226062756227</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -10241,22 +10241,22 @@
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>19/11/2031</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1949</t>
+          <t>1917</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226062756227</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>050526110338066</t>
+          <t>050526131349498</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10640,7 +10640,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>050526131349498</t>
+          <t>050526110338066</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10704,7 +10704,7 @@
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>050526110338113</t>
+          <t>050826061104264</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10768,7 +10768,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>050826061104264</t>
+          <t>050526110338113</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10800,7 +10800,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C163" t="inlineStr"/>
@@ -10817,22 +10817,22 @@
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>050526110338081</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
@@ -10881,12 +10881,12 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>27/01/2032</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>050826061104248</t>
+          <t>050526131349514</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>050826061104420</t>
+          <t>050526110338128</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -11073,12 +11073,12 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>27/01/2032</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1986</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>050526110338128</t>
+          <t>050826061104248</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>050526131349514</t>
+          <t>050526131349576</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11184,7 +11184,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C169" t="inlineStr"/>
@@ -11201,22 +11201,22 @@
       <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>050526110338081</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11248,7 +11248,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
@@ -11265,22 +11265,22 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>26/10/2031</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>050826061104420</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>26/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>050526131349482</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>050526131349576</t>
+          <t>050526131349482</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>200226062905996</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226062905996</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1886</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12353,22 +12353,22 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1886</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1949</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12491,12 +12491,12 @@
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1949</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12880,7 +12880,7 @@
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>300726064011887</t>
+          <t>300726064011918</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12944,7 +12944,7 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>300726064011997</t>
+          <t>300726064012543</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -13008,7 +13008,7 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>300726064011903</t>
+          <t>300726064012575</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
@@ -13057,12 +13057,12 @@
       <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/01/2032</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1819</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13072,7 +13072,7 @@
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>300726064012731</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -13136,7 +13136,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>300726064012543</t>
+          <t>300726064011903</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>300726064012981</t>
+          <t>300726064011997</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>300726064012637</t>
+          <t>300726064011950</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>300726064012512</t>
+          <t>300726064012637</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>300726064011668</t>
+          <t>300726064012903</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>300726064012903</t>
+          <t>300726064012512</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>300726064012825</t>
+          <t>300726064011856</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>300726064012575</t>
+          <t>300726064011887</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>300726064012731</t>
+          <t>300726064012981</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13680,7 +13680,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C208" t="inlineStr"/>
@@ -13697,12 +13697,12 @@
       <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
-          <t>20/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1819</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>300726064011856</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>300726064011950</t>
+          <t>300726064011668</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>300726064011918</t>
+          <t>300726064012825</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -18416,7 +18416,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C282" t="inlineStr"/>
@@ -18433,22 +18433,22 @@
       <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1977</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>280726145221681</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -18463,7 +18463,7 @@
       </c>
       <c r="M282" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N282" t="inlineStr">
@@ -18480,7 +18480,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C283" t="inlineStr"/>
@@ -18497,22 +18497,22 @@
       <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>1977</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>280726145221681</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -18527,7 +18527,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N283" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 20/08/2026 08:37:47
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3393,22 +3393,22 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -18480,7 +18480,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C283" t="inlineStr"/>
@@ -18497,22 +18497,22 @@
       <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1977</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>280726145222103</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -18527,7 +18527,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N283" t="inlineStr">
@@ -18544,7 +18544,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C284" t="inlineStr"/>
@@ -18561,22 +18561,22 @@
       <c r="F284" t="inlineStr"/>
       <c r="G284" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>1977</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>280726145222103</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N284" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 20/08/2026 08:50:25
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -720,7 +720,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1965</t>
+          <t>1817</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1965</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -907,12 +907,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -976,7 +976,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1003,12 +1003,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>323</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1867,12 +1867,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1931,12 +1931,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2379,12 +2379,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-006-002</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>120826061048765</t>
+          <t>120826061048718</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2955,12 +2955,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>120826061048718</t>
+          <t>120826061048781</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3019,12 +3019,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>120826061048781</t>
+          <t>120826061048734</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>2698</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-008-002</t>
+          <t>CAL-027-006-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>120826061048750</t>
+          <t>120826061048765</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-008-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>120826061048734</t>
+          <t>120826061048750</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2698</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132439716</t>
+          <t>110226132439794</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130526104519119</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132440388</t>
+          <t>110226132439716</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439763</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132440529</t>
+          <t>130526104519119</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3563,12 +3563,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132439653</t>
+          <t>110226132439685</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132439685</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440482</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3819,12 +3819,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104518994</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3979,12 +3979,12 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>110226132440450</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4203,12 +4203,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132439653</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4299,12 +4299,12 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132440529</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4353,22 +4353,22 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4395,12 +4395,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -4417,22 +4417,22 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130526104518994</t>
+          <t>110226132440388</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4459,12 +4459,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132439607</t>
+          <t>110226132440450</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132440466</t>
+          <t>110226132439778</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,22 +4609,22 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440482</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4737,22 +4737,22 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4875,12 +4875,12 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132439763</t>
+          <t>110226132440466</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4971,12 +4971,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132439607</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132439794</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>110226132439778</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5569,27 +5569,27 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1805</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -5599,7 +5599,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5633,27 +5633,27 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1805</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6017,22 +6017,22 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6081,12 +6081,12 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6209,12 +6209,12 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6401,12 +6401,12 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6667,12 +6667,12 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6795,12 +6795,12 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6815,7 +6815,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6913,22 +6913,22 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -6992,7 +699